<commit_message>
Replace lat/lon with Google Maps route links in company list
Each company now has a clickable driving route from the restaurant.
build_aziende.py fills real driving km/minutes via the Distance Matrix
API when GOOGLE_MAPS_API_KEY is set, and sorts by driving distance.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JM7iB7irnbem4Sqp1rNjCu
</commit_message>
<xml_diff>
--- a/marketing/aziende_10km_arte_bianca.xlsx
+++ b/marketing/aziende_10km_arte_bianca.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Email template NL" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Aziende'!$A$4:$M$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Aziende'!$A$4:$L$57</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -42,11 +42,6 @@
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="000000FF"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <sz val="9"/>
     </font>
     <font>
@@ -63,6 +58,12 @@
     <font>
       <name val="Arial"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="000563C1"/>
+      <sz val="10"/>
+      <u val="single"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -120,44 +121,43 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="3" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="3" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -167,7 +167,7 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -244,21 +244,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Claude</author>
-  </authors>
-  <commentList>
-    <comment ref="B2" authorId="0" shapeId="0">
-      <text>
-        <t>Coordinate stimate dell'indirizzo del ristorante (Hingene/Wintam). Distanze = formula haversine da queste coordinate.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -550,7 +535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M59"/>
+  <dimension ref="A1:L59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -564,8 +549,7 @@
     <col width="36" customWidth="1" min="9" max="9"/>
     <col width="22" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="9" customWidth="1" min="12" max="12"/>
-    <col width="9" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -578,2928 +562,2918 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Origine lat</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="n">
-        <v>51.1095</v>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Origine lon</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="n">
-        <v>4.2935</v>
-      </c>
-      <c r="E2" s="4" t="inlineStr">
+          <t>Partenza:</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Egied De Jonghestraat 165, 2880 Bornem, Belgium</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>Aziende in elenco:</t>
         </is>
       </c>
-      <c r="F2" s="5" t="n">
+      <c r="F2" s="4" t="n">
         <v>53</v>
       </c>
-      <c r="G2" s="4" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>Con email generica:</t>
         </is>
       </c>
-      <c r="H2" s="5" t="n">
+      <c r="H2" s="4" t="n">
         <v>44</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Azienda</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>Settore</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>Indirizzo</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>Comune</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>Distanza (km, linea d'aria)</t>
         </is>
       </c>
-      <c r="G4" s="6" t="inlineStr">
+      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>Dipendenti (FTE/stima)</t>
         </is>
       </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>Nota dipendenti / fonte</t>
         </is>
       </c>
-      <c r="I4" s="6" t="inlineStr">
+      <c r="I4" s="5" t="inlineStr">
         <is>
           <t>Email generica</t>
         </is>
       </c>
-      <c r="J4" s="6" t="inlineStr">
+      <c r="J4" s="5" t="inlineStr">
         <is>
           <t>Email HR generica</t>
         </is>
       </c>
-      <c r="K4" s="6" t="inlineStr">
+      <c r="K4" s="5" t="inlineStr">
         <is>
           <t>Telefono</t>
         </is>
       </c>
-      <c r="L4" s="6" t="inlineStr">
-        <is>
-          <t>Lat</t>
-        </is>
-      </c>
-      <c r="M4" s="6" t="inlineStr">
-        <is>
-          <t>Lon</t>
+      <c r="L4" s="5" t="inlineStr">
+        <is>
+          <t>Percorso Google Maps</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="n">
+      <c r="A5" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>Topfloor</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>Pavimenti/arredo – produzione</t>
         </is>
       </c>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>Lodderstraat 18</t>
         </is>
       </c>
-      <c r="E5" s="7" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>Bornem (Eikevliet)</t>
         </is>
       </c>
-      <c r="F5" s="9" t="n">
+      <c r="F5" s="8" t="n">
         <v>1.9</v>
       </c>
-      <c r="G5" s="10" t="n">
+      <c r="G5" s="9" t="n">
         <v>24</v>
       </c>
-      <c r="H5" s="8" t="inlineStr">
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>24 FTE (companyweb)</t>
         </is>
       </c>
-      <c r="I5" s="7" t="inlineStr">
+      <c r="I5" s="6" t="inlineStr">
         <is>
           <t>info@topfloor.be</t>
         </is>
       </c>
-      <c r="J5" s="7" t="inlineStr"/>
-      <c r="K5" s="7" t="inlineStr">
+      <c r="J5" s="6" t="inlineStr"/>
+      <c r="K5" s="6" t="inlineStr">
         <is>
           <t>+32 3 889 38 15</t>
         </is>
       </c>
-      <c r="L5" s="11" t="n">
-        <v>51.0935</v>
-      </c>
-      <c r="M5" s="11" t="n">
-        <v>4.2835</v>
+      <c r="L5" s="10" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="n">
+      <c r="A6" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>BMW Group Belux (BMW Belgium Luxembourg)</t>
         </is>
       </c>
-      <c r="C6" s="13" t="inlineStr">
+      <c r="C6" s="12" t="inlineStr">
         <is>
           <t>Automotive – sede Benelux</t>
         </is>
       </c>
-      <c r="D6" s="12" t="inlineStr">
+      <c r="D6" s="11" t="inlineStr">
         <is>
           <t>Lodderstraat 16</t>
         </is>
       </c>
-      <c r="E6" s="12" t="inlineStr">
+      <c r="E6" s="11" t="inlineStr">
         <is>
           <t>Bornem (Eikevliet)</t>
         </is>
       </c>
-      <c r="F6" s="14" t="n">
+      <c r="F6" s="13" t="n">
         <v>1.9</v>
       </c>
-      <c r="G6" s="15" t="n">
+      <c r="G6" s="14" t="n">
         <v>170</v>
       </c>
-      <c r="H6" s="13" t="inlineStr">
+      <c r="H6" s="12" t="inlineStr">
         <is>
           <t>170 FTE (bilancio); ~600 dal 2027 con nuova sede</t>
         </is>
       </c>
-      <c r="I6" s="12" t="inlineStr">
+      <c r="I6" s="11" t="inlineStr">
         <is>
           <t>contact.be@bmw.be</t>
         </is>
       </c>
-      <c r="J6" s="12" t="inlineStr"/>
-      <c r="K6" s="12" t="inlineStr">
+      <c r="J6" s="11" t="inlineStr"/>
+      <c r="K6" s="11" t="inlineStr">
         <is>
           <t>+32 3 890 50 02</t>
         </is>
       </c>
-      <c r="L6" s="16" t="n">
-        <v>51.0935</v>
-      </c>
-      <c r="M6" s="16" t="n">
-        <v>4.283</v>
+      <c r="L6" s="15" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="n">
+      <c r="A7" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>Vétoquinol Belgium</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>Farmaceutica veterinaria</t>
         </is>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>Galileilaan 11/401</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>Niel</t>
         </is>
       </c>
-      <c r="F7" s="9" t="n">
+      <c r="F7" s="8" t="n">
         <v>3.1</v>
       </c>
-      <c r="G7" s="10" t="n">
+      <c r="G7" s="9" t="n">
         <v>33</v>
       </c>
-      <c r="H7" s="8" t="inlineStr">
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>33 FTE (companyweb)</t>
         </is>
       </c>
-      <c r="I7" s="7" t="inlineStr">
+      <c r="I7" s="6" t="inlineStr">
         <is>
           <t>info.be@vetoquinol.com</t>
         </is>
       </c>
-      <c r="J7" s="7" t="inlineStr"/>
-      <c r="K7" s="7" t="inlineStr">
+      <c r="J7" s="6" t="inlineStr"/>
+      <c r="K7" s="6" t="inlineStr">
         <is>
           <t>+32 3 877 44 34</t>
         </is>
       </c>
-      <c r="L7" s="11" t="n">
-        <v>51.117</v>
-      </c>
-      <c r="M7" s="11" t="n">
-        <v>4.336</v>
+      <c r="L7" s="10" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="n">
+      <c r="A8" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B8" s="12" t="inlineStr">
         <is>
           <t>Neovia Logistics</t>
         </is>
       </c>
-      <c r="C8" s="13" t="inlineStr">
+      <c r="C8" s="12" t="inlineStr">
         <is>
           <t>Logistica</t>
         </is>
       </c>
-      <c r="D8" s="12" t="inlineStr">
+      <c r="D8" s="11" t="inlineStr">
         <is>
           <t>Schoonmansveld 1</t>
         </is>
       </c>
-      <c r="E8" s="12" t="inlineStr">
+      <c r="E8" s="11" t="inlineStr">
         <is>
           <t>Puurs-Sint-Amands</t>
         </is>
       </c>
-      <c r="F8" s="14" t="n">
+      <c r="F8" s="13" t="n">
         <v>3.1</v>
       </c>
-      <c r="G8" s="15" t="n">
+      <c r="G8" s="14" t="n">
         <v>189</v>
       </c>
-      <c r="H8" s="13" t="inlineStr">
+      <c r="H8" s="12" t="inlineStr">
         <is>
           <t>189 FTE (companyweb)</t>
         </is>
       </c>
-      <c r="I8" s="12" t="inlineStr">
+      <c r="I8" s="11" t="inlineStr">
         <is>
           <t>reception@neovialogistics.com</t>
         </is>
       </c>
-      <c r="J8" s="12" t="inlineStr"/>
-      <c r="K8" s="12" t="inlineStr">
+      <c r="J8" s="11" t="inlineStr"/>
+      <c r="K8" s="11" t="inlineStr">
         <is>
           <t>+32 2 263 46 11</t>
         </is>
       </c>
-      <c r="L8" s="16" t="n">
-        <v>51.083</v>
-      </c>
-      <c r="M8" s="16" t="n">
-        <v>4.309</v>
+      <c r="L8" s="15" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="n">
+      <c r="A9" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>DSV Solutions Puurs</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>Logistica – magazzino</t>
         </is>
       </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>Schoonmansveld 34</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr">
+      <c r="E9" s="6" t="inlineStr">
         <is>
           <t>Puurs-Sint-Amands</t>
         </is>
       </c>
-      <c r="F9" s="9" t="n">
+      <c r="F9" s="8" t="n">
         <v>3.2</v>
       </c>
-      <c r="G9" s="10" t="n">
+      <c r="G9" s="9" t="n">
         <v>500</v>
       </c>
-      <c r="H9" s="8" t="inlineStr">
+      <c r="H9" s="7" t="inlineStr">
         <is>
           <t>range 500–999 (Gouden Gids, da verificare)</t>
         </is>
       </c>
-      <c r="I9" s="7" t="inlineStr">
+      <c r="I9" s="6" t="inlineStr">
         <is>
           <t>puurs.solutions@be.dsv.com</t>
         </is>
       </c>
-      <c r="J9" s="7" t="inlineStr"/>
-      <c r="K9" s="7" t="inlineStr">
+      <c r="J9" s="6" t="inlineStr"/>
+      <c r="K9" s="6" t="inlineStr">
         <is>
           <t>+32 3 860 35 00</t>
         </is>
       </c>
-      <c r="L9" s="11" t="n">
-        <v>51.0825</v>
-      </c>
-      <c r="M9" s="11" t="n">
-        <v>4.31</v>
+      <c r="L9" s="10" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="n">
+      <c r="A10" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>Transport Robbyns</t>
         </is>
       </c>
-      <c r="C10" s="13" t="inlineStr">
+      <c r="C10" s="12" t="inlineStr">
         <is>
           <t>Trasporti</t>
         </is>
       </c>
-      <c r="D10" s="12" t="inlineStr">
+      <c r="D10" s="11" t="inlineStr">
         <is>
           <t>Schoonmansveld 26</t>
         </is>
       </c>
-      <c r="E10" s="12" t="inlineStr">
+      <c r="E10" s="11" t="inlineStr">
         <is>
           <t>Puurs-Sint-Amands</t>
         </is>
       </c>
-      <c r="F10" s="14" t="n">
+      <c r="F10" s="13" t="n">
         <v>3.3</v>
       </c>
-      <c r="G10" s="15" t="n">
+      <c r="G10" s="14" t="n">
         <v>70</v>
       </c>
-      <c r="H10" s="13" t="inlineStr">
+      <c r="H10" s="12" t="inlineStr">
         <is>
           <t>70 FTE (companyweb)</t>
         </is>
       </c>
-      <c r="I10" s="12" t="inlineStr">
+      <c r="I10" s="11" t="inlineStr">
         <is>
           <t>planning@robbyns.be</t>
         </is>
       </c>
-      <c r="J10" s="12" t="inlineStr"/>
-      <c r="K10" s="12" t="inlineStr">
+      <c r="J10" s="11" t="inlineStr"/>
+      <c r="K10" s="11" t="inlineStr">
         <is>
           <t>+32 3 866 04 21</t>
         </is>
       </c>
-      <c r="L10" s="16" t="n">
-        <v>51.0822</v>
-      </c>
-      <c r="M10" s="16" t="n">
-        <v>4.3105</v>
+      <c r="L10" s="15" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="n">
+      <c r="A11" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>DSV Road + DSV Air &amp; Sea</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>Logistica/spedizioni</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>Schoonmansveld 40</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>Puurs-Sint-Amands</t>
         </is>
       </c>
-      <c r="F11" s="9" t="n">
+      <c r="F11" s="8" t="n">
         <v>3.3</v>
       </c>
-      <c r="G11" s="10" t="n">
+      <c r="G11" s="9" t="n">
         <v>480</v>
       </c>
-      <c r="H11" s="8" t="inlineStr">
+      <c r="H11" s="7" t="inlineStr">
         <is>
           <t>254 + 226 FTE (companyweb)</t>
         </is>
       </c>
-      <c r="I11" s="7" t="inlineStr">
+      <c r="I11" s="6" t="inlineStr">
         <is>
           <t>info.sea@be.dsv.com</t>
         </is>
       </c>
-      <c r="J11" s="7" t="inlineStr"/>
-      <c r="K11" s="7" t="inlineStr">
+      <c r="J11" s="6" t="inlineStr"/>
+      <c r="K11" s="6" t="inlineStr">
         <is>
           <t>+32 3 611 06 00</t>
         </is>
       </c>
-      <c r="L11" s="11" t="n">
-        <v>51.082</v>
-      </c>
-      <c r="M11" s="11" t="n">
-        <v>4.311</v>
+      <c r="L11" s="10" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="n">
+      <c r="A12" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="13" t="inlineStr">
+      <c r="B12" s="12" t="inlineStr">
         <is>
           <t>Groven+</t>
         </is>
       </c>
-      <c r="C12" s="13" t="inlineStr">
+      <c r="C12" s="12" t="inlineStr">
         <is>
           <t>Serramenti/costruzioni</t>
         </is>
       </c>
-      <c r="D12" s="12" t="inlineStr">
+      <c r="D12" s="11" t="inlineStr">
         <is>
           <t>Schoonmansveld 50</t>
         </is>
       </c>
-      <c r="E12" s="12" t="inlineStr">
+      <c r="E12" s="11" t="inlineStr">
         <is>
           <t>Puurs-Sint-Amands</t>
         </is>
       </c>
-      <c r="F12" s="14" t="n">
+      <c r="F12" s="13" t="n">
         <v>3.3</v>
       </c>
-      <c r="G12" s="15" t="n">
+      <c r="G12" s="14" t="n">
         <v>50</v>
       </c>
-      <c r="H12" s="13" t="inlineStr">
+      <c r="H12" s="12" t="inlineStr">
         <is>
           <t>~50 dip.</t>
         </is>
       </c>
-      <c r="I12" s="12" t="inlineStr">
+      <c r="I12" s="11" t="inlineStr">
         <is>
           <t>home@grovenplus.be</t>
         </is>
       </c>
-      <c r="J12" s="12" t="inlineStr"/>
-      <c r="K12" s="12" t="inlineStr">
+      <c r="J12" s="11" t="inlineStr"/>
+      <c r="K12" s="11" t="inlineStr">
         <is>
           <t>+32 3 877 00 44</t>
         </is>
       </c>
-      <c r="L12" s="16" t="n">
-        <v>51.0818</v>
-      </c>
-      <c r="M12" s="16" t="n">
-        <v>4.3115</v>
+      <c r="L12" s="15" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="n">
+      <c r="A13" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>Air Liquide Medical</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
+      <c r="C13" s="7" t="inlineStr">
         <is>
           <t>Gas medicali</t>
         </is>
       </c>
-      <c r="D13" s="7" t="inlineStr">
+      <c r="D13" s="6" t="inlineStr">
         <is>
           <t>Tolhuisstraat 46-48</t>
         </is>
       </c>
-      <c r="E13" s="7" t="inlineStr">
+      <c r="E13" s="6" t="inlineStr">
         <is>
           <t>Schelle</t>
         </is>
       </c>
-      <c r="F13" s="9" t="n">
+      <c r="F13" s="8" t="n">
         <v>3.4</v>
       </c>
-      <c r="G13" s="10" t="n">
+      <c r="G13" s="9" t="n">
         <v>150</v>
       </c>
-      <c r="H13" s="8" t="inlineStr">
+      <c r="H13" s="7" t="inlineStr">
         <is>
           <t>range 100–199 (Gouden Gids)</t>
         </is>
       </c>
-      <c r="I13" s="7" t="inlineStr">
+      <c r="I13" s="6" t="inlineStr">
         <is>
           <t>contact.be@airliquide.com</t>
         </is>
       </c>
-      <c r="J13" s="7" t="inlineStr"/>
-      <c r="K13" s="7" t="inlineStr">
+      <c r="J13" s="6" t="inlineStr"/>
+      <c r="K13" s="6" t="inlineStr">
         <is>
           <t>+32 3 870 84 00</t>
         </is>
       </c>
-      <c r="L13" s="11" t="n">
-        <v>51.127</v>
-      </c>
-      <c r="M13" s="11" t="n">
-        <v>4.334</v>
+      <c r="L13" s="10" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="n">
+      <c r="A14" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="13" t="inlineStr">
+      <c r="B14" s="12" t="inlineStr">
         <is>
           <t>Qualiphar</t>
         </is>
       </c>
-      <c r="C14" s="13" t="inlineStr">
+      <c r="C14" s="12" t="inlineStr">
         <is>
           <t>Farmaceutica/OTC</t>
         </is>
       </c>
-      <c r="D14" s="12" t="inlineStr">
+      <c r="D14" s="11" t="inlineStr">
         <is>
           <t>Rijksweg 9</t>
         </is>
       </c>
-      <c r="E14" s="12" t="inlineStr">
+      <c r="E14" s="11" t="inlineStr">
         <is>
           <t>Bornem</t>
         </is>
       </c>
-      <c r="F14" s="14" t="n">
+      <c r="F14" s="13" t="n">
         <v>3.6</v>
       </c>
-      <c r="G14" s="15" t="n">
+      <c r="G14" s="14" t="n">
         <v>118</v>
       </c>
-      <c r="H14" s="13" t="inlineStr">
+      <c r="H14" s="12" t="inlineStr">
         <is>
           <t>118 dip. (fonte terza, da verificare)</t>
         </is>
       </c>
-      <c r="I14" s="12" t="inlineStr">
+      <c r="I14" s="11" t="inlineStr">
         <is>
           <t>receptie@qualiphar.com</t>
         </is>
       </c>
-      <c r="J14" s="12" t="inlineStr"/>
-      <c r="K14" s="12" t="inlineStr">
+      <c r="J14" s="11" t="inlineStr"/>
+      <c r="K14" s="11" t="inlineStr">
         <is>
           <t>+32 3 889 17 21</t>
         </is>
       </c>
-      <c r="L14" s="16" t="n">
-        <v>51.087</v>
-      </c>
-      <c r="M14" s="16" t="n">
-        <v>4.257</v>
+      <c r="L14" s="15" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="n">
+      <c r="A15" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="8" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>LyondellBasell (A. Schulman Plastics)</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
+      <c r="C15" s="7" t="inlineStr">
         <is>
           <t>Chimica – compound plastici</t>
         </is>
       </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="D15" s="6" t="inlineStr">
         <is>
           <t>Pedro Colomalaan 25</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr">
+      <c r="E15" s="6" t="inlineStr">
         <is>
           <t>Bornem</t>
         </is>
       </c>
-      <c r="F15" s="9" t="n">
+      <c r="F15" s="8" t="n">
         <v>3.6</v>
       </c>
-      <c r="G15" s="10" t="n">
+      <c r="G15" s="9" t="n">
         <v>195</v>
       </c>
-      <c r="H15" s="8" t="inlineStr">
+      <c r="H15" s="7" t="inlineStr">
         <is>
           <t>195 FTE (companyweb)</t>
         </is>
       </c>
-      <c r="I15" s="17" t="inlineStr">
+      <c r="I15" s="16" t="inlineStr">
         <is>
           <t>n.d. (nessuna email generica pubblica)</t>
         </is>
       </c>
-      <c r="J15" s="7" t="inlineStr"/>
-      <c r="K15" s="7" t="inlineStr">
+      <c r="J15" s="6" t="inlineStr"/>
+      <c r="K15" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L15" s="11" t="n">
-        <v>51.09</v>
-      </c>
-      <c r="M15" s="11" t="n">
-        <v>4.252</v>
+      <c r="L15" s="10" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="12" t="n">
+      <c r="A16" s="11" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="13" t="inlineStr">
+      <c r="B16" s="12" t="inlineStr">
         <is>
           <t>Arseus Medical</t>
         </is>
       </c>
-      <c r="C16" s="13" t="inlineStr">
+      <c r="C16" s="12" t="inlineStr">
         <is>
           <t>Forniture medicali</t>
         </is>
       </c>
-      <c r="D16" s="12" t="inlineStr">
+      <c r="D16" s="11" t="inlineStr">
         <is>
           <t>Rijksweg 10</t>
         </is>
       </c>
-      <c r="E16" s="12" t="inlineStr">
+      <c r="E16" s="11" t="inlineStr">
         <is>
           <t>Bornem</t>
         </is>
       </c>
-      <c r="F16" s="14" t="n">
+      <c r="F16" s="13" t="n">
         <v>3.6</v>
       </c>
-      <c r="G16" s="15" t="n">
+      <c r="G16" s="14" t="n">
         <v>66</v>
       </c>
-      <c r="H16" s="13" t="inlineStr">
+      <c r="H16" s="12" t="inlineStr">
         <is>
           <t>66 FTE (Arseus Medical Group, companyweb)</t>
         </is>
       </c>
-      <c r="I16" s="12" t="inlineStr">
+      <c r="I16" s="11" t="inlineStr">
         <is>
           <t>info@arseus-medical.be</t>
         </is>
       </c>
-      <c r="J16" s="12" t="inlineStr"/>
-      <c r="K16" s="12" t="inlineStr">
+      <c r="J16" s="11" t="inlineStr"/>
+      <c r="K16" s="11" t="inlineStr">
         <is>
           <t>+32 800 76 777</t>
         </is>
       </c>
-      <c r="L16" s="16" t="n">
-        <v>51.087</v>
-      </c>
-      <c r="M16" s="16" t="n">
-        <v>4.256</v>
+      <c r="L16" s="15" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="n">
+      <c r="A17" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="8" t="inlineStr">
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>Peleman Industries</t>
         </is>
       </c>
-      <c r="C17" s="8" t="inlineStr">
+      <c r="C17" s="7" t="inlineStr">
         <is>
           <t>Industria – rilegatura/stampa</t>
         </is>
       </c>
-      <c r="D17" s="7" t="inlineStr">
+      <c r="D17" s="6" t="inlineStr">
         <is>
           <t>Rijksweg 7</t>
         </is>
       </c>
-      <c r="E17" s="7" t="inlineStr">
+      <c r="E17" s="6" t="inlineStr">
         <is>
           <t>Puurs-Sint-Amands</t>
         </is>
       </c>
-      <c r="F17" s="9" t="n">
+      <c r="F17" s="8" t="n">
         <v>3.6</v>
       </c>
-      <c r="G17" s="10" t="n">
+      <c r="G17" s="9" t="n">
         <v>84</v>
       </c>
-      <c r="H17" s="8" t="inlineStr">
+      <c r="H17" s="7" t="inlineStr">
         <is>
           <t>84 FTE (companyweb)</t>
         </is>
       </c>
-      <c r="I17" s="7" t="inlineStr">
+      <c r="I17" s="6" t="inlineStr">
         <is>
           <t>info.be@peleman.com</t>
         </is>
       </c>
-      <c r="J17" s="7" t="inlineStr"/>
-      <c r="K17" s="7" t="inlineStr">
+      <c r="J17" s="6" t="inlineStr"/>
+      <c r="K17" s="6" t="inlineStr">
         <is>
           <t>+32 3 889 32 41</t>
         </is>
       </c>
-      <c r="L17" s="11" t="n">
-        <v>51.081</v>
-      </c>
-      <c r="M17" s="11" t="n">
-        <v>4.268</v>
+      <c r="L17" s="10" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="12" t="n">
+      <c r="A18" s="11" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="13" t="inlineStr">
+      <c r="B18" s="12" t="inlineStr">
         <is>
           <t>Lonza Capsules (Capsugel Belgium)</t>
         </is>
       </c>
-      <c r="C18" s="13" t="inlineStr">
+      <c r="C18" s="12" t="inlineStr">
         <is>
           <t>Farmaceutica – capsule</t>
         </is>
       </c>
-      <c r="D18" s="12" t="inlineStr">
+      <c r="D18" s="11" t="inlineStr">
         <is>
           <t>Rijksweg 11</t>
         </is>
       </c>
-      <c r="E18" s="12" t="inlineStr">
+      <c r="E18" s="11" t="inlineStr">
         <is>
           <t>Bornem</t>
         </is>
       </c>
-      <c r="F18" s="14" t="n">
+      <c r="F18" s="13" t="n">
         <v>3.7</v>
       </c>
-      <c r="G18" s="15" t="n">
+      <c r="G18" s="14" t="n">
         <v>474</v>
       </c>
-      <c r="H18" s="13" t="inlineStr">
+      <c r="H18" s="12" t="inlineStr">
         <is>
           <t>474 FTE (companyweb)</t>
         </is>
       </c>
-      <c r="I18" s="18" t="inlineStr">
+      <c r="I18" s="17" t="inlineStr">
         <is>
           <t>n.d. (nessuna email generica pubblica)</t>
         </is>
       </c>
-      <c r="J18" s="12" t="inlineStr"/>
-      <c r="K18" s="12" t="inlineStr">
+      <c r="J18" s="11" t="inlineStr"/>
+      <c r="K18" s="11" t="inlineStr">
         <is>
           <t>+32 3 890 05 11</t>
         </is>
       </c>
-      <c r="L18" s="16" t="n">
-        <v>51.086</v>
-      </c>
-      <c r="M18" s="16" t="n">
-        <v>4.256</v>
+      <c r="L18" s="15" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="n">
+      <c r="A19" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="8" t="inlineStr">
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>AZ Rivierenland – campus Bornem</t>
         </is>
       </c>
-      <c r="C19" s="8" t="inlineStr">
+      <c r="C19" s="7" t="inlineStr">
         <is>
           <t>Ospedale</t>
         </is>
       </c>
-      <c r="D19" s="7" t="inlineStr">
+      <c r="D19" s="6" t="inlineStr">
         <is>
           <t>Kasteelstraat 23</t>
         </is>
       </c>
-      <c r="E19" s="7" t="inlineStr">
+      <c r="E19" s="6" t="inlineStr">
         <is>
           <t>Bornem</t>
         </is>
       </c>
-      <c r="F19" s="9" t="n">
+      <c r="F19" s="8" t="n">
         <v>3.8</v>
       </c>
-      <c r="G19" s="10" t="n">
+      <c r="G19" s="9" t="n">
         <v>1500</v>
       </c>
-      <c r="H19" s="8" t="inlineStr">
+      <c r="H19" s="7" t="inlineStr">
         <is>
           <t>stima, tutti i campus (Bornem/Rumst/Willebroek)</t>
         </is>
       </c>
-      <c r="I19" s="7" t="inlineStr">
+      <c r="I19" s="6" t="inlineStr">
         <is>
           <t>info@azr.be</t>
         </is>
       </c>
-      <c r="J19" s="7" t="inlineStr"/>
-      <c r="K19" s="7" t="inlineStr">
+      <c r="J19" s="6" t="inlineStr"/>
+      <c r="K19" s="6" t="inlineStr">
         <is>
           <t>+32 3 880 90 11</t>
         </is>
       </c>
-      <c r="L19" s="11" t="n">
-        <v>51.0975</v>
-      </c>
-      <c r="M19" s="11" t="n">
-        <v>4.243</v>
+      <c r="L19" s="10" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="12" t="n">
+      <c r="A20" s="11" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="13" t="inlineStr">
+      <c r="B20" s="12" t="inlineStr">
         <is>
           <t>European Master Batch (Sioen Chemicals)</t>
         </is>
       </c>
-      <c r="C20" s="13" t="inlineStr">
+      <c r="C20" s="12" t="inlineStr">
         <is>
           <t>Chimica – masterbatch</t>
         </is>
       </c>
-      <c r="D20" s="12" t="inlineStr">
+      <c r="D20" s="11" t="inlineStr">
         <is>
           <t>Rijksweg 15</t>
         </is>
       </c>
-      <c r="E20" s="12" t="inlineStr">
+      <c r="E20" s="11" t="inlineStr">
         <is>
           <t>Bornem</t>
         </is>
       </c>
-      <c r="F20" s="14" t="n">
+      <c r="F20" s="13" t="n">
         <v>3.8</v>
       </c>
-      <c r="G20" s="15" t="n">
+      <c r="G20" s="14" t="n">
         <v>108</v>
       </c>
-      <c r="H20" s="13" t="inlineStr">
+      <c r="H20" s="12" t="inlineStr">
         <is>
           <t>108 FTE (companyweb)</t>
         </is>
       </c>
-      <c r="I20" s="12" t="inlineStr">
+      <c r="I20" s="11" t="inlineStr">
         <is>
           <t>info@sioenchemicals.com</t>
         </is>
       </c>
-      <c r="J20" s="12" t="inlineStr"/>
-      <c r="K20" s="12" t="inlineStr">
+      <c r="J20" s="11" t="inlineStr"/>
+      <c r="K20" s="11" t="inlineStr">
         <is>
           <t>+32 3 890 64 00</t>
         </is>
       </c>
-      <c r="L20" s="16" t="n">
-        <v>51.085</v>
-      </c>
-      <c r="M20" s="16" t="n">
-        <v>4.255</v>
+      <c r="L20" s="15" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="n">
+      <c r="A21" s="6" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="8" t="inlineStr">
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>Olympus Belgium</t>
         </is>
       </c>
-      <c r="C21" s="8" t="inlineStr">
+      <c r="C21" s="7" t="inlineStr">
         <is>
           <t>Dispositivi medici/ottica</t>
         </is>
       </c>
-      <c r="D21" s="7" t="inlineStr">
+      <c r="D21" s="6" t="inlineStr">
         <is>
           <t>Gansbroekstraat 70</t>
         </is>
       </c>
-      <c r="E21" s="7" t="inlineStr">
+      <c r="E21" s="6" t="inlineStr">
         <is>
           <t>Puurs-Sint-Amands</t>
         </is>
       </c>
-      <c r="F21" s="9" t="n">
+      <c r="F21" s="8" t="n">
         <v>3.8</v>
       </c>
-      <c r="G21" s="10" t="n">
+      <c r="G21" s="9" t="n">
         <v>48</v>
       </c>
-      <c r="H21" s="8" t="inlineStr">
+      <c r="H21" s="7" t="inlineStr">
         <is>
           <t>48 FTE (companyweb)</t>
         </is>
       </c>
-      <c r="I21" s="17" t="inlineStr">
+      <c r="I21" s="16" t="inlineStr">
         <is>
           <t>n.d. (solo modulo web olympus.be)</t>
         </is>
       </c>
-      <c r="J21" s="7" t="inlineStr"/>
-      <c r="K21" s="7" t="inlineStr">
+      <c r="J21" s="6" t="inlineStr"/>
+      <c r="K21" s="6" t="inlineStr">
         <is>
           <t>+32 3 870 58 00</t>
         </is>
       </c>
-      <c r="L21" s="11" t="n">
-        <v>51.075</v>
-      </c>
-      <c r="M21" s="11" t="n">
-        <v>4.298</v>
+      <c r="L21" s="10" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="12" t="n">
+      <c r="A22" s="11" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="13" t="inlineStr">
+      <c r="B22" s="12" t="inlineStr">
         <is>
           <t>Smurfit Westrock Bornem</t>
         </is>
       </c>
-      <c r="C22" s="13" t="inlineStr">
+      <c r="C22" s="12" t="inlineStr">
         <is>
           <t>Packaging</t>
         </is>
       </c>
-      <c r="D22" s="12" t="inlineStr">
+      <c r="D22" s="11" t="inlineStr">
         <is>
           <t>Rijksweg 18</t>
         </is>
       </c>
-      <c r="E22" s="12" t="inlineStr">
+      <c r="E22" s="11" t="inlineStr">
         <is>
           <t>Bornem</t>
         </is>
       </c>
-      <c r="F22" s="14" t="n">
+      <c r="F22" s="13" t="n">
         <v>3.9</v>
       </c>
-      <c r="G22" s="15" t="n">
+      <c r="G22" s="14" t="n">
         <v>151</v>
       </c>
-      <c r="H22" s="13" t="inlineStr">
+      <c r="H22" s="12" t="inlineStr">
         <is>
           <t>151 FTE (companyweb)</t>
         </is>
       </c>
-      <c r="I22" s="12" t="inlineStr">
+      <c r="I22" s="11" t="inlineStr">
         <is>
           <t>onthaal.bornem@multipkg.com</t>
         </is>
       </c>
-      <c r="J22" s="12" t="inlineStr"/>
-      <c r="K22" s="12" t="inlineStr">
+      <c r="J22" s="11" t="inlineStr"/>
+      <c r="K22" s="11" t="inlineStr">
         <is>
           <t>+32 3 889 68 11</t>
         </is>
       </c>
-      <c r="L22" s="16" t="n">
-        <v>51.085</v>
-      </c>
-      <c r="M22" s="16" t="n">
-        <v>4.254</v>
+      <c r="L22" s="15" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="7" t="n">
+      <c r="A23" s="6" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="8" t="inlineStr">
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>Pfizer Manufacturing Belgium</t>
         </is>
       </c>
-      <c r="C23" s="8" t="inlineStr">
+      <c r="C23" s="7" t="inlineStr">
         <is>
           <t>Farmaceutica – produzione</t>
         </is>
       </c>
-      <c r="D23" s="7" t="inlineStr">
+      <c r="D23" s="6" t="inlineStr">
         <is>
           <t>Rijksweg 12</t>
         </is>
       </c>
-      <c r="E23" s="7" t="inlineStr">
+      <c r="E23" s="6" t="inlineStr">
         <is>
           <t>Puurs-Sint-Amands</t>
         </is>
       </c>
-      <c r="F23" s="9" t="n">
+      <c r="F23" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="G23" s="10" t="n">
+      <c r="G23" s="9" t="n">
         <v>4021</v>
       </c>
-      <c r="H23" s="8" t="inlineStr">
+      <c r="H23" s="7" t="inlineStr">
         <is>
           <t>4.021 FTE (companyweb) – maggior datore di lavoro della zona</t>
         </is>
       </c>
-      <c r="I23" s="17" t="inlineStr">
+      <c r="I23" s="16" t="inlineStr">
         <is>
           <t>n.d. (nessuna email generica pubblica)</t>
         </is>
       </c>
-      <c r="J23" s="7" t="inlineStr"/>
-      <c r="K23" s="7" t="inlineStr">
+      <c r="J23" s="6" t="inlineStr"/>
+      <c r="K23" s="6" t="inlineStr">
         <is>
           <t>+32 3 890 92 11</t>
         </is>
       </c>
-      <c r="L23" s="11" t="n">
-        <v>51.0786</v>
-      </c>
-      <c r="M23" s="11" t="n">
-        <v>4.264</v>
+      <c r="L23" s="10" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="12" t="n">
+      <c r="A24" s="11" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="13" t="inlineStr">
+      <c r="B24" s="12" t="inlineStr">
         <is>
           <t>Novartis Manufacturing</t>
         </is>
       </c>
-      <c r="C24" s="13" t="inlineStr">
+      <c r="C24" s="12" t="inlineStr">
         <is>
           <t>Farmaceutica – produzione</t>
         </is>
       </c>
-      <c r="D24" s="12" t="inlineStr">
+      <c r="D24" s="11" t="inlineStr">
         <is>
           <t>Rijksweg 14</t>
         </is>
       </c>
-      <c r="E24" s="12" t="inlineStr">
+      <c r="E24" s="11" t="inlineStr">
         <is>
           <t>Puurs-Sint-Amands</t>
         </is>
       </c>
-      <c r="F24" s="14" t="n">
+      <c r="F24" s="13" t="n">
         <v>4.3</v>
       </c>
-      <c r="G24" s="15" t="n">
+      <c r="G24" s="14" t="n">
         <v>980</v>
       </c>
-      <c r="H24" s="13" t="inlineStr">
+      <c r="H24" s="12" t="inlineStr">
         <is>
           <t>980 FTE (companyweb)</t>
         </is>
       </c>
-      <c r="I24" s="18" t="inlineStr">
+      <c r="I24" s="17" t="inlineStr">
         <is>
           <t>n.d. (nessuna email generica pubblica)</t>
         </is>
       </c>
-      <c r="J24" s="12" t="inlineStr"/>
-      <c r="K24" s="12" t="inlineStr">
+      <c r="J24" s="11" t="inlineStr"/>
+      <c r="K24" s="11" t="inlineStr">
         <is>
           <t>+32 3 890 28 00</t>
         </is>
       </c>
-      <c r="L24" s="16" t="n">
-        <v>51.077</v>
-      </c>
-      <c r="M24" s="16" t="n">
-        <v>4.26</v>
+      <c r="L24" s="15" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="7" t="n">
+      <c r="A25" s="6" t="n">
         <v>21</v>
       </c>
-      <c r="B25" s="8" t="inlineStr">
+      <c r="B25" s="7" t="inlineStr">
         <is>
           <t>Lamifil</t>
         </is>
       </c>
-      <c r="C25" s="8" t="inlineStr">
+      <c r="C25" s="7" t="inlineStr">
         <is>
           <t>Industria – cavi/fili</t>
         </is>
       </c>
-      <c r="D25" s="7" t="inlineStr">
+      <c r="D25" s="6" t="inlineStr">
         <is>
           <t>Frederic Sheidlaan</t>
         </is>
       </c>
-      <c r="E25" s="7" t="inlineStr">
+      <c r="E25" s="6" t="inlineStr">
         <is>
           <t>Hemiksem</t>
         </is>
       </c>
-      <c r="F25" s="9" t="n">
+      <c r="F25" s="8" t="n">
         <v>4.3</v>
       </c>
-      <c r="G25" s="10" t="n">
+      <c r="G25" s="9" t="n">
         <v>224</v>
       </c>
-      <c r="H25" s="8" t="inlineStr">
+      <c r="H25" s="7" t="inlineStr">
         <is>
           <t>224 FTE (companyweb)</t>
         </is>
       </c>
-      <c r="I25" s="7" t="inlineStr">
+      <c r="I25" s="6" t="inlineStr">
         <is>
           <t>info@lamifil.be</t>
         </is>
       </c>
-      <c r="J25" s="7" t="inlineStr"/>
-      <c r="K25" s="7" t="inlineStr">
+      <c r="J25" s="6" t="inlineStr"/>
+      <c r="K25" s="6" t="inlineStr">
         <is>
           <t>+32 3 870 06 11</t>
         </is>
       </c>
-      <c r="L25" s="11" t="n">
-        <v>51.1395</v>
-      </c>
-      <c r="M25" s="11" t="n">
-        <v>4.333</v>
+      <c r="L25" s="10" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="12" t="n">
+      <c r="A26" s="11" t="n">
         <v>22</v>
       </c>
-      <c r="B26" s="13" t="inlineStr">
+      <c r="B26" s="12" t="inlineStr">
         <is>
           <t>Studio 100 (sede centrale)</t>
         </is>
       </c>
-      <c r="C26" s="13" t="inlineStr">
+      <c r="C26" s="12" t="inlineStr">
         <is>
           <t>Media/intrattenimento</t>
         </is>
       </c>
-      <c r="D26" s="12" t="inlineStr">
+      <c r="D26" s="11" t="inlineStr">
         <is>
           <t>Halfstraat 80</t>
         </is>
       </c>
-      <c r="E26" s="12" t="inlineStr">
+      <c r="E26" s="11" t="inlineStr">
         <is>
           <t>Schelle</t>
         </is>
       </c>
-      <c r="F26" s="14" t="n">
+      <c r="F26" s="13" t="n">
         <v>4.5</v>
       </c>
-      <c r="G26" s="15" t="n">
+      <c r="G26" s="14" t="n">
         <v>169</v>
       </c>
-      <c r="H26" s="13" t="inlineStr">
+      <c r="H26" s="12" t="inlineStr">
         <is>
           <t>169 FTE (2025)</t>
         </is>
       </c>
-      <c r="I26" s="12" t="inlineStr">
+      <c r="I26" s="11" t="inlineStr">
         <is>
           <t>info@studio100.be</t>
         </is>
       </c>
-      <c r="J26" s="12" t="inlineStr"/>
-      <c r="K26" s="12" t="inlineStr">
+      <c r="J26" s="11" t="inlineStr"/>
+      <c r="K26" s="11" t="inlineStr">
         <is>
           <t>+32 3 877 60 35</t>
         </is>
       </c>
-      <c r="L26" s="16" t="n">
-        <v>51.131</v>
-      </c>
-      <c r="M26" s="16" t="n">
-        <v>4.348</v>
+      <c r="L26" s="15" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="7" t="n">
+      <c r="A27" s="6" t="n">
         <v>23</v>
       </c>
-      <c r="B27" s="8" t="inlineStr">
+      <c r="B27" s="7" t="inlineStr">
         <is>
           <t>Atlas Copco Rental Europe</t>
         </is>
       </c>
-      <c r="C27" s="8" t="inlineStr">
+      <c r="C27" s="7" t="inlineStr">
         <is>
           <t>Noleggio attrezzature</t>
         </is>
       </c>
-      <c r="D27" s="7" t="inlineStr">
+      <c r="D27" s="6" t="inlineStr">
         <is>
           <t>Industrieweg 1F</t>
         </is>
       </c>
-      <c r="E27" s="7" t="inlineStr">
+      <c r="E27" s="6" t="inlineStr">
         <is>
           <t>Boom</t>
         </is>
       </c>
-      <c r="F27" s="9" t="n">
+      <c r="F27" s="8" t="n">
         <v>4.5</v>
       </c>
-      <c r="G27" s="10" t="n">
+      <c r="G27" s="9" t="n">
         <v>123</v>
       </c>
-      <c r="H27" s="8" t="inlineStr">
+      <c r="H27" s="7" t="inlineStr">
         <is>
           <t>123 FTE (companyweb)</t>
         </is>
       </c>
-      <c r="I27" s="7" t="inlineStr">
+      <c r="I27" s="6" t="inlineStr">
         <is>
           <t>rental.belgium@atlascopco.com</t>
         </is>
       </c>
-      <c r="J27" s="7" t="inlineStr"/>
-      <c r="K27" s="7" t="inlineStr">
+      <c r="J27" s="6" t="inlineStr"/>
+      <c r="K27" s="6" t="inlineStr">
         <is>
           <t>+32 3 401 67 67</t>
         </is>
       </c>
-      <c r="L27" s="11" t="n">
-        <v>51.097</v>
-      </c>
-      <c r="M27" s="11" t="n">
-        <v>4.355</v>
+      <c r="L27" s="10" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="12" t="n">
+      <c r="A28" s="11" t="n">
         <v>24</v>
       </c>
-      <c r="B28" s="13" t="inlineStr">
+      <c r="B28" s="12" t="inlineStr">
         <is>
           <t>Besix Infra</t>
         </is>
       </c>
-      <c r="C28" s="13" t="inlineStr">
+      <c r="C28" s="12" t="inlineStr">
         <is>
           <t>Costruzioni/infrastrutture</t>
         </is>
       </c>
-      <c r="D28" s="12" t="inlineStr">
+      <c r="D28" s="11" t="inlineStr">
         <is>
           <t>Steenwinkelstraat 640</t>
         </is>
       </c>
-      <c r="E28" s="12" t="inlineStr">
+      <c r="E28" s="11" t="inlineStr">
         <is>
           <t>Schelle</t>
         </is>
       </c>
-      <c r="F28" s="14" t="n">
+      <c r="F28" s="13" t="n">
         <v>4.6</v>
       </c>
-      <c r="G28" s="15" t="n">
+      <c r="G28" s="14" t="n">
         <v>323</v>
       </c>
-      <c r="H28" s="13" t="inlineStr">
+      <c r="H28" s="12" t="inlineStr">
         <is>
           <t>323 FTE (companyweb)</t>
         </is>
       </c>
-      <c r="I28" s="12" t="inlineStr">
+      <c r="I28" s="11" t="inlineStr">
         <is>
           <t>besixinfra@besix.com</t>
         </is>
       </c>
-      <c r="J28" s="12" t="inlineStr"/>
-      <c r="K28" s="12" t="inlineStr">
+      <c r="J28" s="11" t="inlineStr"/>
+      <c r="K28" s="11" t="inlineStr">
         <is>
           <t>+32 3 870 79 70</t>
         </is>
       </c>
-      <c r="L28" s="16" t="n">
-        <v>51.119</v>
-      </c>
-      <c r="M28" s="16" t="n">
-        <v>4.357</v>
+      <c r="L28" s="15" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="7" t="n">
+      <c r="A29" s="6" t="n">
         <v>25</v>
       </c>
-      <c r="B29" s="8" t="inlineStr">
+      <c r="B29" s="7" t="inlineStr">
         <is>
           <t>Pelican Rouge</t>
         </is>
       </c>
-      <c r="C29" s="8" t="inlineStr">
+      <c r="C29" s="7" t="inlineStr">
         <is>
           <t>Caffè/vending</t>
         </is>
       </c>
-      <c r="D29" s="7" t="inlineStr">
+      <c r="D29" s="6" t="inlineStr">
         <is>
           <t>Industrieweg 10a</t>
         </is>
       </c>
-      <c r="E29" s="7" t="inlineStr">
+      <c r="E29" s="6" t="inlineStr">
         <is>
           <t>Boom</t>
         </is>
       </c>
-      <c r="F29" s="9" t="n">
+      <c r="F29" s="8" t="n">
         <v>4.6</v>
       </c>
-      <c r="G29" s="10" t="n">
+      <c r="G29" s="9" t="n">
         <v>344</v>
       </c>
-      <c r="H29" s="8" t="inlineStr">
+      <c r="H29" s="7" t="inlineStr">
         <is>
           <t>344 FTE (companyweb)</t>
         </is>
       </c>
-      <c r="I29" s="17" t="inlineStr">
+      <c r="I29" s="16" t="inlineStr">
         <is>
           <t>n.d. (nessuna email generica pubblica)</t>
         </is>
       </c>
-      <c r="J29" s="7" t="inlineStr"/>
-      <c r="K29" s="7" t="inlineStr">
+      <c r="J29" s="6" t="inlineStr"/>
+      <c r="K29" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L29" s="11" t="n">
-        <v>51.0965</v>
-      </c>
-      <c r="M29" s="11" t="n">
-        <v>4.356</v>
+      <c r="L29" s="10" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="12" t="n">
+      <c r="A30" s="11" t="n">
         <v>26</v>
       </c>
-      <c r="B30" s="13" t="inlineStr">
+      <c r="B30" s="12" t="inlineStr">
         <is>
           <t>Wolf Oil Corporation</t>
         </is>
       </c>
-      <c r="C30" s="13" t="inlineStr">
+      <c r="C30" s="12" t="inlineStr">
         <is>
           <t>Lubrificanti</t>
         </is>
       </c>
-      <c r="D30" s="12" t="inlineStr">
+      <c r="D30" s="11" t="inlineStr">
         <is>
           <t>Georges Gilliotstraat 52</t>
         </is>
       </c>
-      <c r="E30" s="12" t="inlineStr">
+      <c r="E30" s="11" t="inlineStr">
         <is>
           <t>Hemiksem</t>
         </is>
       </c>
-      <c r="F30" s="14" t="n">
+      <c r="F30" s="13" t="n">
         <v>4.6</v>
       </c>
-      <c r="G30" s="15" t="n">
+      <c r="G30" s="14" t="n">
         <v>75</v>
       </c>
-      <c r="H30" s="13" t="inlineStr">
+      <c r="H30" s="12" t="inlineStr">
         <is>
           <t>75 FTE (companyweb)</t>
         </is>
       </c>
-      <c r="I30" s="12" t="inlineStr">
+      <c r="I30" s="11" t="inlineStr">
         <is>
           <t>info@wolfoil.com</t>
         </is>
       </c>
-      <c r="J30" s="12" t="inlineStr"/>
-      <c r="K30" s="12" t="inlineStr">
+      <c r="J30" s="11" t="inlineStr"/>
+      <c r="K30" s="11" t="inlineStr">
         <is>
           <t>+32 3 870 00 00</t>
         </is>
       </c>
-      <c r="L30" s="16" t="n">
-        <v>51.14</v>
-      </c>
-      <c r="M30" s="16" t="n">
-        <v>4.338</v>
+      <c r="L30" s="15" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="7" t="n">
+      <c r="A31" s="6" t="n">
         <v>27</v>
       </c>
-      <c r="B31" s="8" t="inlineStr">
+      <c r="B31" s="7" t="inlineStr">
         <is>
           <t>Champion Chemicals</t>
         </is>
       </c>
-      <c r="C31" s="8" t="inlineStr">
+      <c r="C31" s="7" t="inlineStr">
         <is>
           <t>Lubrificanti</t>
         </is>
       </c>
-      <c r="D31" s="7" t="inlineStr">
+      <c r="D31" s="6" t="inlineStr">
         <is>
           <t>Georges Gilliotstraat 52</t>
         </is>
       </c>
-      <c r="E31" s="7" t="inlineStr">
+      <c r="E31" s="6" t="inlineStr">
         <is>
           <t>Hemiksem</t>
         </is>
       </c>
-      <c r="F31" s="9" t="n">
+      <c r="F31" s="8" t="n">
         <v>4.6</v>
       </c>
-      <c r="G31" s="10" t="n">
+      <c r="G31" s="9" t="n">
         <v>85</v>
       </c>
-      <c r="H31" s="8" t="inlineStr">
+      <c r="H31" s="7" t="inlineStr">
         <is>
           <t>85 FTE (companyweb)</t>
         </is>
       </c>
-      <c r="I31" s="7" t="inlineStr">
+      <c r="I31" s="6" t="inlineStr">
         <is>
           <t>info@championlubes.com</t>
         </is>
       </c>
-      <c r="J31" s="7" t="inlineStr"/>
-      <c r="K31" s="7" t="inlineStr">
+      <c r="J31" s="6" t="inlineStr"/>
+      <c r="K31" s="6" t="inlineStr">
         <is>
           <t>+32 3 870 00 20</t>
         </is>
       </c>
-      <c r="L31" s="11" t="n">
-        <v>51.14</v>
-      </c>
-      <c r="M31" s="11" t="n">
-        <v>4.3385</v>
+      <c r="L31" s="10" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="12" t="n">
+      <c r="A32" s="11" t="n">
         <v>28</v>
       </c>
-      <c r="B32" s="13" t="inlineStr">
+      <c r="B32" s="12" t="inlineStr">
         <is>
           <t>Bakker Belgium (Greenyard)</t>
         </is>
       </c>
-      <c r="C32" s="13" t="inlineStr">
+      <c r="C32" s="12" t="inlineStr">
         <is>
           <t>Ortofrutta – logistica</t>
         </is>
       </c>
-      <c r="D32" s="12" t="inlineStr">
+      <c r="D32" s="11" t="inlineStr">
         <is>
           <t>Industrieweg 16</t>
         </is>
       </c>
-      <c r="E32" s="12" t="inlineStr">
+      <c r="E32" s="11" t="inlineStr">
         <is>
           <t>Boom</t>
         </is>
       </c>
-      <c r="F32" s="14" t="n">
+      <c r="F32" s="13" t="n">
         <v>4.7</v>
       </c>
-      <c r="G32" s="15" t="n">
+      <c r="G32" s="14" t="n">
         <v>151</v>
       </c>
-      <c r="H32" s="13" t="inlineStr">
+      <c r="H32" s="12" t="inlineStr">
         <is>
           <t>151 FTE (companyweb)</t>
         </is>
       </c>
-      <c r="I32" s="12" t="inlineStr">
+      <c r="I32" s="11" t="inlineStr">
         <is>
           <t>info@bakkerbelgium.be</t>
         </is>
       </c>
-      <c r="J32" s="12" t="inlineStr"/>
-      <c r="K32" s="12" t="inlineStr">
+      <c r="J32" s="11" t="inlineStr"/>
+      <c r="K32" s="11" t="inlineStr">
         <is>
           <t>+32 3 808 84 00</t>
         </is>
       </c>
-      <c r="L32" s="16" t="n">
-        <v>51.096</v>
-      </c>
-      <c r="M32" s="16" t="n">
-        <v>4.357</v>
+      <c r="L32" s="15" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="7" t="n">
+      <c r="A33" s="6" t="n">
         <v>29</v>
       </c>
-      <c r="B33" s="8" t="inlineStr">
+      <c r="B33" s="7" t="inlineStr">
         <is>
           <t>BD – Becton Dickinson Distribution Center</t>
         </is>
       </c>
-      <c r="C33" s="8" t="inlineStr">
+      <c r="C33" s="7" t="inlineStr">
         <is>
           <t>Medtech – distribuzione</t>
         </is>
       </c>
-      <c r="D33" s="7" t="inlineStr">
+      <c r="D33" s="6" t="inlineStr">
         <is>
           <t>Laagstraat 57 (IZ TTS)</t>
         </is>
       </c>
-      <c r="E33" s="7" t="inlineStr">
+      <c r="E33" s="6" t="inlineStr">
         <is>
           <t>Temse</t>
         </is>
       </c>
-      <c r="F33" s="9" t="n">
+      <c r="F33" s="8" t="n">
         <v>5.3</v>
       </c>
-      <c r="G33" s="10" t="n">
+      <c r="G33" s="9" t="n">
         <v>434</v>
       </c>
-      <c r="H33" s="8" t="inlineStr">
+      <c r="H33" s="7" t="inlineStr">
         <is>
           <t>434 FTE (companyweb)</t>
         </is>
       </c>
-      <c r="I33" s="7" t="inlineStr">
+      <c r="I33" s="6" t="inlineStr">
         <is>
           <t>info.benelux@bd.com</t>
         </is>
       </c>
-      <c r="J33" s="7" t="inlineStr"/>
-      <c r="K33" s="7" t="inlineStr">
+      <c r="J33" s="6" t="inlineStr"/>
+      <c r="K33" s="6" t="inlineStr">
         <is>
           <t>+32 3 710 32 06</t>
         </is>
       </c>
-      <c r="L33" s="11" t="n">
-        <v>51.134</v>
-      </c>
-      <c r="M33" s="11" t="n">
-        <v>4.229</v>
+      <c r="L33" s="10" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="12" t="n">
+      <c r="A34" s="11" t="n">
         <v>30</v>
       </c>
-      <c r="B34" s="13" t="inlineStr">
+      <c r="B34" s="12" t="inlineStr">
         <is>
           <t>Multi.Engineering</t>
         </is>
       </c>
-      <c r="C34" s="13" t="inlineStr">
+      <c r="C34" s="12" t="inlineStr">
         <is>
           <t>Engineering</t>
         </is>
       </c>
-      <c r="D34" s="12" t="inlineStr">
+      <c r="D34" s="11" t="inlineStr">
         <is>
           <t>Orlaylaan 10 (IZ TTS)</t>
         </is>
       </c>
-      <c r="E34" s="12" t="inlineStr">
+      <c r="E34" s="11" t="inlineStr">
         <is>
           <t>Temse</t>
         </is>
       </c>
-      <c r="F34" s="14" t="n">
+      <c r="F34" s="13" t="n">
         <v>5.4</v>
       </c>
-      <c r="G34" s="15" t="n">
+      <c r="G34" s="14" t="n">
         <v>54</v>
       </c>
-      <c r="H34" s="13" t="inlineStr">
+      <c r="H34" s="12" t="inlineStr">
         <is>
           <t>54 FTE (companyweb)</t>
         </is>
       </c>
-      <c r="I34" s="12" t="inlineStr">
+      <c r="I34" s="11" t="inlineStr">
         <is>
           <t>info.temse@multi.engineering</t>
         </is>
       </c>
-      <c r="J34" s="12" t="inlineStr"/>
-      <c r="K34" s="12" t="inlineStr">
+      <c r="J34" s="11" t="inlineStr"/>
+      <c r="K34" s="11" t="inlineStr">
         <is>
           <t>+32 3 710 58 10</t>
         </is>
       </c>
-      <c r="L34" s="16" t="n">
-        <v>51.1345</v>
-      </c>
-      <c r="M34" s="16" t="n">
-        <v>4.228</v>
+      <c r="L34" s="15" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="7" t="n">
+      <c r="A35" s="6" t="n">
         <v>31</v>
       </c>
-      <c r="B35" s="8" t="inlineStr">
+      <c r="B35" s="7" t="inlineStr">
         <is>
           <t>De Meyer NV</t>
         </is>
       </c>
-      <c r="C35" s="8" t="inlineStr">
+      <c r="C35" s="7" t="inlineStr">
         <is>
           <t>Meccanica/engineering</t>
         </is>
       </c>
-      <c r="D35" s="7" t="inlineStr">
+      <c r="D35" s="6" t="inlineStr">
         <is>
           <t>Frank Van Dyckelaan 28</t>
         </is>
       </c>
-      <c r="E35" s="7" t="inlineStr">
+      <c r="E35" s="6" t="inlineStr">
         <is>
           <t>Temse</t>
         </is>
       </c>
-      <c r="F35" s="9" t="n">
+      <c r="F35" s="8" t="n">
         <v>5.4</v>
       </c>
-      <c r="G35" s="10" t="n">
+      <c r="G35" s="9" t="n">
         <v>130</v>
       </c>
-      <c r="H35" s="8" t="inlineStr">
+      <c r="H35" s="7" t="inlineStr">
         <is>
           <t>~130 dip. (sito aziendale)</t>
         </is>
       </c>
-      <c r="I35" s="7" t="inlineStr">
+      <c r="I35" s="6" t="inlineStr">
         <is>
           <t>info@demeyer.be</t>
         </is>
       </c>
-      <c r="J35" s="7" t="inlineStr"/>
-      <c r="K35" s="7" t="inlineStr">
+      <c r="J35" s="6" t="inlineStr"/>
+      <c r="K35" s="6" t="inlineStr">
         <is>
           <t>+32 3 766 33 33</t>
         </is>
       </c>
-      <c r="L35" s="11" t="n">
-        <v>51.1258</v>
-      </c>
-      <c r="M35" s="11" t="n">
-        <v>4.221</v>
+      <c r="L35" s="10" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="12" t="n">
+      <c r="A36" s="11" t="n">
         <v>32</v>
       </c>
-      <c r="B36" s="13" t="inlineStr">
+      <c r="B36" s="12" t="inlineStr">
         <is>
           <t>C-Metal (gruppo Cordeel)</t>
         </is>
       </c>
-      <c r="C36" s="13" t="inlineStr">
+      <c r="C36" s="12" t="inlineStr">
         <is>
           <t>Carpenteria metallica</t>
         </is>
       </c>
-      <c r="D36" s="12" t="inlineStr">
+      <c r="D36" s="11" t="inlineStr">
         <is>
           <t>Frank Van Dyckelaan 19A</t>
         </is>
       </c>
-      <c r="E36" s="12" t="inlineStr">
+      <c r="E36" s="11" t="inlineStr">
         <is>
           <t>Temse</t>
         </is>
       </c>
-      <c r="F36" s="14" t="n">
+      <c r="F36" s="13" t="n">
         <v>5.4</v>
       </c>
-      <c r="G36" s="15" t="n">
+      <c r="G36" s="14" t="n">
         <v>51</v>
       </c>
-      <c r="H36" s="13" t="inlineStr">
+      <c r="H36" s="12" t="inlineStr">
         <is>
           <t>51 FTE (companyweb)</t>
         </is>
       </c>
-      <c r="I36" s="12" t="inlineStr">
+      <c r="I36" s="11" t="inlineStr">
         <is>
           <t>info@c-metal.eu</t>
         </is>
       </c>
-      <c r="J36" s="12" t="inlineStr"/>
-      <c r="K36" s="12" t="inlineStr">
+      <c r="J36" s="11" t="inlineStr"/>
+      <c r="K36" s="11" t="inlineStr">
         <is>
           <t>+32 3 710 55 62</t>
         </is>
       </c>
-      <c r="L36" s="16" t="n">
-        <v>51.1255</v>
-      </c>
-      <c r="M36" s="16" t="n">
-        <v>4.2205</v>
+      <c r="L36" s="15" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="7" t="n">
+      <c r="A37" s="6" t="n">
         <v>33</v>
       </c>
-      <c r="B37" s="8" t="inlineStr">
+      <c r="B37" s="7" t="inlineStr">
         <is>
           <t>Cordeel (sede centrale)</t>
         </is>
       </c>
-      <c r="C37" s="8" t="inlineStr">
+      <c r="C37" s="7" t="inlineStr">
         <is>
           <t>Costruzioni</t>
         </is>
       </c>
-      <c r="D37" s="7" t="inlineStr">
+      <c r="D37" s="6" t="inlineStr">
         <is>
           <t>Frank Van Dyckelaan 15</t>
         </is>
       </c>
-      <c r="E37" s="7" t="inlineStr">
+      <c r="E37" s="6" t="inlineStr">
         <is>
           <t>Temse</t>
         </is>
       </c>
-      <c r="F37" s="9" t="n">
+      <c r="F37" s="8" t="n">
         <v>5.4</v>
       </c>
-      <c r="G37" s="10" t="n">
+      <c r="G37" s="9" t="n">
         <v>199</v>
       </c>
-      <c r="H37" s="8" t="inlineStr">
+      <c r="H37" s="7" t="inlineStr">
         <is>
           <t>199 FTE Cordeel Zetel Temse (companyweb)</t>
         </is>
       </c>
-      <c r="I37" s="7" t="inlineStr">
+      <c r="I37" s="6" t="inlineStr">
         <is>
           <t>info@cordeel.eu</t>
         </is>
       </c>
-      <c r="J37" s="7" t="inlineStr"/>
-      <c r="K37" s="7" t="inlineStr">
+      <c r="J37" s="6" t="inlineStr"/>
+      <c r="K37" s="6" t="inlineStr">
         <is>
           <t>+32 3 710 55 00</t>
         </is>
       </c>
-      <c r="L37" s="11" t="n">
-        <v>51.1255</v>
-      </c>
-      <c r="M37" s="11" t="n">
-        <v>4.22</v>
+      <c r="L37" s="10" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="12" t="n">
+      <c r="A38" s="11" t="n">
         <v>34</v>
       </c>
-      <c r="B38" s="13" t="inlineStr">
+      <c r="B38" s="12" t="inlineStr">
         <is>
           <t>Modemakers Fashion</t>
         </is>
       </c>
-      <c r="C38" s="13" t="inlineStr">
+      <c r="C38" s="12" t="inlineStr">
         <is>
           <t>Moda – distribuzione</t>
         </is>
       </c>
-      <c r="D38" s="12" t="inlineStr">
+      <c r="D38" s="11" t="inlineStr">
         <is>
           <t>Kapelanielaan 17 (IZ TTS)</t>
         </is>
       </c>
-      <c r="E38" s="12" t="inlineStr">
+      <c r="E38" s="11" t="inlineStr">
         <is>
           <t>Temse</t>
         </is>
       </c>
-      <c r="F38" s="14" t="n">
+      <c r="F38" s="13" t="n">
         <v>5.4</v>
       </c>
-      <c r="G38" s="15" t="n">
+      <c r="G38" s="14" t="n">
         <v>35</v>
       </c>
-      <c r="H38" s="13" t="inlineStr">
+      <c r="H38" s="12" t="inlineStr">
         <is>
           <t>35 FTE (companyweb)</t>
         </is>
       </c>
-      <c r="I38" s="12" t="inlineStr">
+      <c r="I38" s="11" t="inlineStr">
         <is>
           <t>info@modemakers.be</t>
         </is>
       </c>
-      <c r="J38" s="12" t="inlineStr"/>
-      <c r="K38" s="12" t="inlineStr">
+      <c r="J38" s="11" t="inlineStr"/>
+      <c r="K38" s="11" t="inlineStr">
         <is>
           <t>+32 3 886 59 02</t>
         </is>
       </c>
-      <c r="L38" s="16" t="n">
-        <v>51.135</v>
-      </c>
-      <c r="M38" s="16" t="n">
-        <v>4.227</v>
+      <c r="L38" s="15" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="7" t="n">
+      <c r="A39" s="6" t="n">
         <v>35</v>
       </c>
-      <c r="B39" s="8" t="inlineStr">
+      <c r="B39" s="7" t="inlineStr">
         <is>
           <t>RCT Stevedoring</t>
         </is>
       </c>
-      <c r="C39" s="8" t="inlineStr">
+      <c r="C39" s="7" t="inlineStr">
         <is>
           <t>Logistica portuale</t>
         </is>
       </c>
-      <c r="D39" s="7" t="inlineStr">
+      <c r="D39" s="6" t="inlineStr">
         <is>
           <t>Boomsesteenweg 180</t>
         </is>
       </c>
-      <c r="E39" s="7" t="inlineStr">
+      <c r="E39" s="6" t="inlineStr">
         <is>
           <t>Willebroek</t>
         </is>
       </c>
-      <c r="F39" s="9" t="n">
+      <c r="F39" s="8" t="n">
         <v>5.9</v>
       </c>
-      <c r="G39" s="10" t="n">
+      <c r="G39" s="9" t="n">
         <v>15</v>
       </c>
-      <c r="H39" s="8" t="inlineStr">
+      <c r="H39" s="7" t="inlineStr">
         <is>
           <t>15 FTE (companyweb)</t>
         </is>
       </c>
-      <c r="I39" s="7" t="inlineStr">
+      <c r="I39" s="6" t="inlineStr">
         <is>
           <t>info@rct-stevedoring.com</t>
         </is>
       </c>
-      <c r="J39" s="7" t="inlineStr"/>
-      <c r="K39" s="7" t="inlineStr">
+      <c r="J39" s="6" t="inlineStr"/>
+      <c r="K39" s="6" t="inlineStr">
         <is>
           <t>+32 3 886 37 11</t>
         </is>
       </c>
-      <c r="L39" s="11" t="n">
-        <v>51.075</v>
-      </c>
-      <c r="M39" s="11" t="n">
-        <v>4.357</v>
+      <c r="L39" s="10" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="12" t="n">
+      <c r="A40" s="11" t="n">
         <v>36</v>
       </c>
-      <c r="B40" s="13" t="inlineStr">
+      <c r="B40" s="12" t="inlineStr">
         <is>
           <t>Ceva Logistics Belgium</t>
         </is>
       </c>
-      <c r="C40" s="13" t="inlineStr">
+      <c r="C40" s="12" t="inlineStr">
         <is>
           <t>Logistica</t>
         </is>
       </c>
-      <c r="D40" s="12" t="inlineStr">
+      <c r="D40" s="11" t="inlineStr">
         <is>
           <t>Koningin Astridlaan 12</t>
         </is>
       </c>
-      <c r="E40" s="12" t="inlineStr">
+      <c r="E40" s="11" t="inlineStr">
         <is>
           <t>Willebroek</t>
         </is>
       </c>
-      <c r="F40" s="14" t="n">
+      <c r="F40" s="13" t="n">
         <v>6.3</v>
       </c>
-      <c r="G40" s="15" t="n">
+      <c r="G40" s="14" t="n">
         <v>723</v>
       </c>
-      <c r="H40" s="13" t="inlineStr">
+      <c r="H40" s="12" t="inlineStr">
         <is>
           <t>723 FTE (companyweb)</t>
         </is>
       </c>
-      <c r="I40" s="12" t="inlineStr">
+      <c r="I40" s="11" t="inlineStr">
         <is>
           <t>receptie.willebroek@cevalogistics.com</t>
         </is>
       </c>
-      <c r="J40" s="12" t="inlineStr"/>
-      <c r="K40" s="12" t="inlineStr">
+      <c r="J40" s="11" t="inlineStr"/>
+      <c r="K40" s="11" t="inlineStr">
         <is>
           <t>+32 3 860 45 00</t>
         </is>
       </c>
-      <c r="L40" s="16" t="n">
-        <v>51.068</v>
-      </c>
-      <c r="M40" s="16" t="n">
-        <v>4.355</v>
+      <c r="L40" s="15" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="7" t="n">
+      <c r="A41" s="6" t="n">
         <v>37</v>
       </c>
-      <c r="B41" s="8" t="inlineStr">
+      <c r="B41" s="7" t="inlineStr">
         <is>
           <t>Redwire Space</t>
         </is>
       </c>
-      <c r="C41" s="8" t="inlineStr">
+      <c r="C41" s="7" t="inlineStr">
         <is>
           <t>Aerospazio</t>
         </is>
       </c>
-      <c r="D41" s="7" t="inlineStr">
+      <c r="D41" s="6" t="inlineStr">
         <is>
           <t>Hogenakkerhoekstraat 9</t>
         </is>
       </c>
-      <c r="E41" s="7" t="inlineStr">
+      <c r="E41" s="6" t="inlineStr">
         <is>
           <t>Kruibeke</t>
         </is>
       </c>
-      <c r="F41" s="9" t="n">
+      <c r="F41" s="8" t="n">
         <v>6.3</v>
       </c>
-      <c r="G41" s="10" t="n">
+      <c r="G41" s="9" t="n">
         <v>124</v>
       </c>
-      <c r="H41" s="8" t="inlineStr">
+      <c r="H41" s="7" t="inlineStr">
         <is>
           <t>124 FTE (companyweb)</t>
         </is>
       </c>
-      <c r="I41" s="17" t="inlineStr">
+      <c r="I41" s="16" t="inlineStr">
         <is>
           <t>n.d. (nessuna email generica pubblica)</t>
         </is>
       </c>
-      <c r="J41" s="7" t="inlineStr"/>
-      <c r="K41" s="7" t="inlineStr">
+      <c r="J41" s="6" t="inlineStr"/>
+      <c r="K41" s="6" t="inlineStr">
         <is>
           <t>+32 3 250 14 14</t>
         </is>
       </c>
-      <c r="L41" s="11" t="n">
-        <v>51.166</v>
-      </c>
-      <c r="M41" s="11" t="n">
-        <v>4.305</v>
+      <c r="L41" s="10" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="12" t="n">
+      <c r="A42" s="11" t="n">
         <v>38</v>
       </c>
-      <c r="B42" s="13" t="inlineStr">
+      <c r="B42" s="12" t="inlineStr">
         <is>
           <t>Elscolab</t>
         </is>
       </c>
-      <c r="C42" s="13" t="inlineStr">
+      <c r="C42" s="12" t="inlineStr">
         <is>
           <t>Strumentazione laboratorio</t>
         </is>
       </c>
-      <c r="D42" s="12" t="inlineStr">
+      <c r="D42" s="11" t="inlineStr">
         <is>
           <t>Hogenakkerhoekstraat 14</t>
         </is>
       </c>
-      <c r="E42" s="12" t="inlineStr">
+      <c r="E42" s="11" t="inlineStr">
         <is>
           <t>Kruibeke</t>
         </is>
       </c>
-      <c r="F42" s="14" t="n">
+      <c r="F42" s="13" t="n">
         <v>6.3</v>
       </c>
-      <c r="G42" s="15" t="n">
+      <c r="G42" s="14" t="n">
         <v>34</v>
       </c>
-      <c r="H42" s="13" t="inlineStr">
+      <c r="H42" s="12" t="inlineStr">
         <is>
           <t>34 FTE (companyweb)</t>
         </is>
       </c>
-      <c r="I42" s="12" t="inlineStr">
+      <c r="I42" s="11" t="inlineStr">
         <is>
           <t>contact@elscolab.com</t>
         </is>
       </c>
-      <c r="J42" s="12" t="inlineStr"/>
-      <c r="K42" s="12" t="inlineStr">
+      <c r="J42" s="11" t="inlineStr"/>
+      <c r="K42" s="11" t="inlineStr">
         <is>
           <t>+32 3 250 15 70</t>
         </is>
       </c>
-      <c r="L42" s="16" t="n">
-        <v>51.1661</v>
-      </c>
-      <c r="M42" s="16" t="n">
-        <v>4.3052</v>
+      <c r="L42" s="15" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="7" t="n">
+      <c r="A43" s="6" t="n">
         <v>39</v>
       </c>
-      <c r="B43" s="8" t="inlineStr">
+      <c r="B43" s="7" t="inlineStr">
         <is>
           <t>Verhaert</t>
         </is>
       </c>
-      <c r="C43" s="8" t="inlineStr">
+      <c r="C43" s="7" t="inlineStr">
         <is>
           <t>Innovazione/product design</t>
         </is>
       </c>
-      <c r="D43" s="7" t="inlineStr">
+      <c r="D43" s="6" t="inlineStr">
         <is>
           <t>Hogenakkerhoekstraat 21</t>
         </is>
       </c>
-      <c r="E43" s="7" t="inlineStr">
+      <c r="E43" s="6" t="inlineStr">
         <is>
           <t>Kruibeke</t>
         </is>
       </c>
-      <c r="F43" s="9" t="n">
+      <c r="F43" s="8" t="n">
         <v>6.4</v>
       </c>
-      <c r="G43" s="10" t="n">
+      <c r="G43" s="9" t="n">
         <v>68</v>
       </c>
-      <c r="H43" s="8" t="inlineStr">
+      <c r="H43" s="7" t="inlineStr">
         <is>
           <t>68 FTE (companyweb)</t>
         </is>
       </c>
-      <c r="I43" s="7" t="inlineStr">
+      <c r="I43" s="6" t="inlineStr">
         <is>
           <t>info@verhaert.com</t>
         </is>
       </c>
-      <c r="J43" s="7" t="inlineStr"/>
-      <c r="K43" s="7" t="inlineStr">
+      <c r="J43" s="6" t="inlineStr"/>
+      <c r="K43" s="6" t="inlineStr">
         <is>
           <t>+32 3 250 19 00</t>
         </is>
       </c>
-      <c r="L43" s="11" t="n">
-        <v>51.1662</v>
-      </c>
-      <c r="M43" s="11" t="n">
-        <v>4.3055</v>
+      <c r="L43" s="10" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="12" t="n">
+      <c r="A44" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="B44" s="13" t="inlineStr">
+      <c r="B44" s="12" t="inlineStr">
         <is>
           <t>Distrilog Group</t>
         </is>
       </c>
-      <c r="C44" s="13" t="inlineStr">
+      <c r="C44" s="12" t="inlineStr">
         <is>
           <t>Logistica</t>
         </is>
       </c>
-      <c r="D44" s="12" t="inlineStr">
+      <c r="D44" s="11" t="inlineStr">
         <is>
           <t>Koningin Astridlaan 14</t>
         </is>
       </c>
-      <c r="E44" s="12" t="inlineStr">
+      <c r="E44" s="11" t="inlineStr">
         <is>
           <t>Willebroek</t>
         </is>
       </c>
-      <c r="F44" s="14" t="n">
+      <c r="F44" s="13" t="n">
         <v>6.4</v>
       </c>
-      <c r="G44" s="15" t="n">
+      <c r="G44" s="14" t="n">
         <v>563</v>
       </c>
-      <c r="H44" s="13" t="inlineStr">
+      <c r="H44" s="12" t="inlineStr">
         <is>
           <t>563 FTE (companyweb)</t>
         </is>
       </c>
-      <c r="I44" s="12" t="inlineStr">
+      <c r="I44" s="11" t="inlineStr">
         <is>
           <t>info@distrilog.be</t>
         </is>
       </c>
-      <c r="J44" s="12" t="inlineStr">
+      <c r="J44" s="11" t="inlineStr">
         <is>
           <t>personeel@distrilog.be</t>
         </is>
       </c>
-      <c r="K44" s="12" t="inlineStr">
+      <c r="K44" s="11" t="inlineStr">
         <is>
           <t>+32 3 897 19 90</t>
         </is>
       </c>
-      <c r="L44" s="16" t="n">
-        <v>51.0675</v>
-      </c>
-      <c r="M44" s="16" t="n">
-        <v>4.3555</v>
+      <c r="L44" s="15" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="7" t="n">
+      <c r="A45" s="6" t="n">
         <v>41</v>
       </c>
-      <c r="B45" s="8" t="inlineStr">
+      <c r="B45" s="7" t="inlineStr">
         <is>
           <t>Grundfos Bellux</t>
         </is>
       </c>
-      <c r="C45" s="8" t="inlineStr">
+      <c r="C45" s="7" t="inlineStr">
         <is>
           <t>Pompe – vendita</t>
         </is>
       </c>
-      <c r="D45" s="7" t="inlineStr">
+      <c r="D45" s="6" t="inlineStr">
         <is>
           <t>Boomsesteenweg 81-83</t>
         </is>
       </c>
-      <c r="E45" s="7" t="inlineStr">
+      <c r="E45" s="6" t="inlineStr">
         <is>
           <t>Aartselaar</t>
         </is>
       </c>
-      <c r="F45" s="9" t="n">
+      <c r="F45" s="8" t="n">
         <v>6.4</v>
       </c>
-      <c r="G45" s="10" t="n">
+      <c r="G45" s="9" t="n">
         <v>75</v>
       </c>
-      <c r="H45" s="8" t="inlineStr">
+      <c r="H45" s="7" t="inlineStr">
         <is>
           <t>range 50–99</t>
         </is>
       </c>
-      <c r="I45" s="7" t="inlineStr">
+      <c r="I45" s="6" t="inlineStr">
         <is>
           <t>infobellux@grundfos.com</t>
         </is>
       </c>
-      <c r="J45" s="7" t="inlineStr"/>
-      <c r="K45" s="7" t="inlineStr">
+      <c r="J45" s="6" t="inlineStr"/>
+      <c r="K45" s="6" t="inlineStr">
         <is>
           <t>+32 3 870 73 00</t>
         </is>
       </c>
-      <c r="L45" s="11" t="n">
-        <v>51.134</v>
-      </c>
-      <c r="M45" s="11" t="n">
-        <v>4.376</v>
+      <c r="L45" s="10" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="12" t="n">
+      <c r="A46" s="11" t="n">
         <v>42</v>
       </c>
-      <c r="B46" s="13" t="inlineStr">
+      <c r="B46" s="12" t="inlineStr">
         <is>
           <t>Toolstation Belgium (sede)</t>
         </is>
       </c>
-      <c r="C46" s="13" t="inlineStr">
+      <c r="C46" s="12" t="inlineStr">
         <is>
           <t>Retail utensili</t>
         </is>
       </c>
-      <c r="D46" s="12" t="inlineStr">
+      <c r="D46" s="11" t="inlineStr">
         <is>
           <t>Boomsesteenweg 58A</t>
         </is>
       </c>
-      <c r="E46" s="12" t="inlineStr">
+      <c r="E46" s="11" t="inlineStr">
         <is>
           <t>Aartselaar</t>
         </is>
       </c>
-      <c r="F46" s="14" t="n">
+      <c r="F46" s="13" t="n">
         <v>6.5</v>
       </c>
-      <c r="G46" s="15" t="n">
+      <c r="G46" s="14" t="n">
         <v>84</v>
       </c>
-      <c r="H46" s="13" t="inlineStr">
+      <c r="H46" s="12" t="inlineStr">
         <is>
           <t>84 FTE (companyweb)</t>
         </is>
       </c>
-      <c r="I46" s="12" t="inlineStr">
+      <c r="I46" s="11" t="inlineStr">
         <is>
           <t>info@toolstation.be</t>
         </is>
       </c>
-      <c r="J46" s="12" t="inlineStr"/>
-      <c r="K46" s="12" t="inlineStr">
+      <c r="J46" s="11" t="inlineStr"/>
+      <c r="K46" s="11" t="inlineStr">
         <is>
           <t>078 05 00 96</t>
         </is>
       </c>
-      <c r="L46" s="16" t="n">
-        <v>51.136</v>
-      </c>
-      <c r="M46" s="16" t="n">
-        <v>4.377</v>
+      <c r="L46" s="15" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="7" t="n">
+      <c r="A47" s="6" t="n">
         <v>43</v>
       </c>
-      <c r="B47" s="8" t="inlineStr">
+      <c r="B47" s="7" t="inlineStr">
         <is>
           <t>Keppel Seghers Belgium</t>
         </is>
       </c>
-      <c r="C47" s="8" t="inlineStr">
+      <c r="C47" s="7" t="inlineStr">
         <is>
           <t>Engineering ambientale</t>
         </is>
       </c>
-      <c r="D47" s="7" t="inlineStr">
+      <c r="D47" s="6" t="inlineStr">
         <is>
           <t>Hoofd 1</t>
         </is>
       </c>
-      <c r="E47" s="7" t="inlineStr">
+      <c r="E47" s="6" t="inlineStr">
         <is>
           <t>Willebroek</t>
         </is>
       </c>
-      <c r="F47" s="9" t="n">
+      <c r="F47" s="8" t="n">
         <v>7</v>
       </c>
-      <c r="G47" s="10" t="n">
+      <c r="G47" s="9" t="n">
         <v>117</v>
       </c>
-      <c r="H47" s="8" t="inlineStr">
+      <c r="H47" s="7" t="inlineStr">
         <is>
           <t>117 FTE (companyweb)</t>
         </is>
       </c>
-      <c r="I47" s="7" t="inlineStr">
+      <c r="I47" s="6" t="inlineStr">
         <is>
           <t>info.keppelseghers@keppel.com</t>
         </is>
       </c>
-      <c r="J47" s="7" t="inlineStr"/>
-      <c r="K47" s="7" t="inlineStr">
+      <c r="J47" s="6" t="inlineStr"/>
+      <c r="K47" s="6" t="inlineStr">
         <is>
           <t>+32 3 880 77 00</t>
         </is>
       </c>
-      <c r="L47" s="11" t="n">
-        <v>51.064</v>
-      </c>
-      <c r="M47" s="11" t="n">
-        <v>4.362</v>
+      <c r="L47" s="10" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="12" t="n">
+      <c r="A48" s="11" t="n">
         <v>44</v>
       </c>
-      <c r="B48" s="13" t="inlineStr">
+      <c r="B48" s="12" t="inlineStr">
         <is>
           <t>Tesla Belgium</t>
         </is>
       </c>
-      <c r="C48" s="13" t="inlineStr">
+      <c r="C48" s="12" t="inlineStr">
         <is>
           <t>Automotive – sede/service</t>
         </is>
       </c>
-      <c r="D48" s="12" t="inlineStr">
+      <c r="D48" s="11" t="inlineStr">
         <is>
           <t>Boomsesteenweg 8</t>
         </is>
       </c>
-      <c r="E48" s="12" t="inlineStr">
+      <c r="E48" s="11" t="inlineStr">
         <is>
           <t>Aartselaar</t>
         </is>
       </c>
-      <c r="F48" s="14" t="n">
+      <c r="F48" s="13" t="n">
         <v>7</v>
       </c>
-      <c r="G48" s="15" t="n">
+      <c r="G48" s="14" t="n">
         <v>231</v>
       </c>
-      <c r="H48" s="13" t="inlineStr">
+      <c r="H48" s="12" t="inlineStr">
         <is>
           <t>231 FTE (companyweb)</t>
         </is>
       </c>
-      <c r="I48" s="18" t="inlineStr">
+      <c r="I48" s="17" t="inlineStr">
         <is>
           <t>n.d. (nessuna email generica pubblica)</t>
         </is>
       </c>
-      <c r="J48" s="12" t="inlineStr"/>
-      <c r="K48" s="12" t="inlineStr">
+      <c r="J48" s="11" t="inlineStr"/>
+      <c r="K48" s="11" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L48" s="16" t="n">
-        <v>51.142</v>
-      </c>
-      <c r="M48" s="16" t="n">
-        <v>4.38</v>
+      <c r="L48" s="15" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="7" t="n">
+      <c r="A49" s="6" t="n">
         <v>45</v>
       </c>
-      <c r="B49" s="8" t="inlineStr">
+      <c r="B49" s="7" t="inlineStr">
         <is>
           <t>TTC Trade &amp; Transport Corporation</t>
         </is>
       </c>
-      <c r="C49" s="8" t="inlineStr">
+      <c r="C49" s="7" t="inlineStr">
         <is>
           <t>Trasporti</t>
         </is>
       </c>
-      <c r="D49" s="7" t="inlineStr">
+      <c r="D49" s="6" t="inlineStr">
         <is>
           <t>Kasteleinsstraat 21</t>
         </is>
       </c>
-      <c r="E49" s="7" t="inlineStr">
+      <c r="E49" s="6" t="inlineStr">
         <is>
           <t>Kruibeke</t>
         </is>
       </c>
-      <c r="F49" s="9" t="n">
+      <c r="F49" s="8" t="n">
         <v>7</v>
       </c>
-      <c r="G49" s="10" t="n">
+      <c r="G49" s="9" t="n">
         <v>233</v>
       </c>
-      <c r="H49" s="8" t="inlineStr">
+      <c r="H49" s="7" t="inlineStr">
         <is>
           <t>233 FTE (companyweb)</t>
         </is>
       </c>
-      <c r="I49" s="7" t="inlineStr">
+      <c r="I49" s="6" t="inlineStr">
         <is>
           <t>administratie@ttctransport.be</t>
         </is>
       </c>
-      <c r="J49" s="7" t="inlineStr"/>
-      <c r="K49" s="7" t="inlineStr">
+      <c r="J49" s="6" t="inlineStr"/>
+      <c r="K49" s="6" t="inlineStr">
         <is>
           <t>+32 3 252 20 80</t>
         </is>
       </c>
-      <c r="L49" s="11" t="n">
-        <v>51.172</v>
-      </c>
-      <c r="M49" s="11" t="n">
-        <v>4.31</v>
+      <c r="L49" s="10" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="12" t="n">
+      <c r="A50" s="11" t="n">
         <v>46</v>
       </c>
-      <c r="B50" s="13" t="inlineStr">
+      <c r="B50" s="12" t="inlineStr">
         <is>
           <t>Belcar</t>
         </is>
       </c>
-      <c r="C50" s="13" t="inlineStr">
+      <c r="C50" s="12" t="inlineStr">
         <is>
           <t>Noleggio/servizi auto</t>
         </is>
       </c>
-      <c r="D50" s="12" t="inlineStr">
+      <c r="D50" s="11" t="inlineStr">
         <is>
           <t>Bist 12</t>
         </is>
       </c>
-      <c r="E50" s="12" t="inlineStr">
+      <c r="E50" s="11" t="inlineStr">
         <is>
           <t>Aartselaar</t>
         </is>
       </c>
-      <c r="F50" s="14" t="n">
+      <c r="F50" s="13" t="n">
         <v>7.3</v>
       </c>
-      <c r="G50" s="15" t="n">
+      <c r="G50" s="14" t="n">
         <v>86</v>
       </c>
-      <c r="H50" s="13" t="inlineStr">
+      <c r="H50" s="12" t="inlineStr">
         <is>
           <t>86 FTE (companyweb)</t>
         </is>
       </c>
-      <c r="I50" s="12" t="inlineStr">
+      <c r="I50" s="11" t="inlineStr">
         <is>
           <t>info@belcar.be</t>
         </is>
       </c>
-      <c r="J50" s="12" t="inlineStr"/>
-      <c r="K50" s="12" t="inlineStr">
+      <c r="J50" s="11" t="inlineStr"/>
+      <c r="K50" s="11" t="inlineStr">
         <is>
           <t>+32 3 870 81 30</t>
         </is>
       </c>
-      <c r="L50" s="16" t="n">
-        <v>51.137</v>
-      </c>
-      <c r="M50" s="16" t="n">
-        <v>4.388</v>
+      <c r="L50" s="15" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="7" t="n">
+      <c r="A51" s="6" t="n">
         <v>47</v>
       </c>
-      <c r="B51" s="8" t="inlineStr">
+      <c r="B51" s="7" t="inlineStr">
         <is>
           <t>Fero Group</t>
         </is>
       </c>
-      <c r="C51" s="8" t="inlineStr">
+      <c r="C51" s="7" t="inlineStr">
         <is>
           <t>Segnaletica/costruzioni</t>
         </is>
       </c>
-      <c r="D51" s="7" t="inlineStr">
+      <c r="D51" s="6" t="inlineStr">
         <is>
           <t>Jozef De Blockstraat 81</t>
         </is>
       </c>
-      <c r="E51" s="7" t="inlineStr">
+      <c r="E51" s="6" t="inlineStr">
         <is>
           <t>Willebroek</t>
         </is>
       </c>
-      <c r="F51" s="9" t="n">
+      <c r="F51" s="8" t="n">
         <v>7.3</v>
       </c>
-      <c r="G51" s="10" t="n">
+      <c r="G51" s="9" t="n">
         <v>174</v>
       </c>
-      <c r="H51" s="8" t="inlineStr">
+      <c r="H51" s="7" t="inlineStr">
         <is>
           <t>174 FTE (companyweb)</t>
         </is>
       </c>
-      <c r="I51" s="7" t="inlineStr">
+      <c r="I51" s="6" t="inlineStr">
         <is>
           <t>info@ferogroup.be</t>
         </is>
       </c>
-      <c r="J51" s="7" t="inlineStr"/>
-      <c r="K51" s="7" t="inlineStr">
+      <c r="J51" s="6" t="inlineStr"/>
+      <c r="K51" s="6" t="inlineStr">
         <is>
           <t>+32 3 288 75 28</t>
         </is>
       </c>
-      <c r="L51" s="11" t="n">
-        <v>51.058</v>
-      </c>
-      <c r="M51" s="11" t="n">
-        <v>4.358</v>
+      <c r="L51" s="10" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="12" t="n">
+      <c r="A52" s="11" t="n">
         <v>48</v>
       </c>
-      <c r="B52" s="13" t="inlineStr">
+      <c r="B52" s="12" t="inlineStr">
         <is>
           <t>ODTH – Opslag en Distributie Ter Haeghe</t>
         </is>
       </c>
-      <c r="C52" s="13" t="inlineStr">
+      <c r="C52" s="12" t="inlineStr">
         <is>
           <t>Logistica chimica</t>
         </is>
       </c>
-      <c r="D52" s="12" t="inlineStr">
+      <c r="D52" s="11" t="inlineStr">
         <is>
           <t>Doelhaagstraat 72</t>
         </is>
       </c>
-      <c r="E52" s="12" t="inlineStr">
+      <c r="E52" s="11" t="inlineStr">
         <is>
           <t>Rumst (Terhagen)</t>
         </is>
       </c>
-      <c r="F52" s="14" t="n">
+      <c r="F52" s="13" t="n">
         <v>7.5</v>
       </c>
-      <c r="G52" s="15" t="n">
+      <c r="G52" s="14" t="n">
         <v>150</v>
       </c>
-      <c r="H52" s="13" t="inlineStr">
+      <c r="H52" s="12" t="inlineStr">
         <is>
           <t>150 FTE (companyweb)</t>
         </is>
       </c>
-      <c r="I52" s="12" t="inlineStr">
+      <c r="I52" s="11" t="inlineStr">
         <is>
           <t>info@odth.be</t>
         </is>
       </c>
-      <c r="J52" s="12" t="inlineStr"/>
-      <c r="K52" s="12" t="inlineStr">
+      <c r="J52" s="11" t="inlineStr"/>
+      <c r="K52" s="11" t="inlineStr">
         <is>
           <t>+32 3 880 72 60</t>
         </is>
       </c>
-      <c r="L52" s="16" t="n">
-        <v>51.087</v>
-      </c>
-      <c r="M52" s="16" t="n">
-        <v>4.395</v>
+      <c r="L52" s="15" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="7" t="n">
+      <c r="A53" s="6" t="n">
         <v>49</v>
       </c>
-      <c r="B53" s="8" t="inlineStr">
+      <c r="B53" s="7" t="inlineStr">
         <is>
           <t>Duvel Moortgat</t>
         </is>
       </c>
-      <c r="C53" s="8" t="inlineStr">
+      <c r="C53" s="7" t="inlineStr">
         <is>
           <t>Birrificio</t>
         </is>
       </c>
-      <c r="D53" s="7" t="inlineStr">
+      <c r="D53" s="6" t="inlineStr">
         <is>
           <t>Breendonk-Dorp 58</t>
         </is>
       </c>
-      <c r="E53" s="7" t="inlineStr">
+      <c r="E53" s="6" t="inlineStr">
         <is>
           <t>Puurs-Sint-Amands (Breendonk)</t>
         </is>
       </c>
-      <c r="F53" s="9" t="n">
+      <c r="F53" s="8" t="n">
         <v>7.6</v>
       </c>
-      <c r="G53" s="10" t="n">
+      <c r="G53" s="9" t="n">
         <v>517</v>
       </c>
-      <c r="H53" s="8" t="inlineStr">
+      <c r="H53" s="7" t="inlineStr">
         <is>
           <t>~517 dip.</t>
         </is>
       </c>
-      <c r="I53" s="7" t="inlineStr">
+      <c r="I53" s="6" t="inlineStr">
         <is>
           <t>info@duvel.be</t>
         </is>
       </c>
-      <c r="J53" s="7" t="inlineStr"/>
-      <c r="K53" s="7" t="inlineStr">
+      <c r="J53" s="6" t="inlineStr"/>
+      <c r="K53" s="6" t="inlineStr">
         <is>
           <t>+32 3 860 94 00</t>
         </is>
       </c>
-      <c r="L53" s="11" t="n">
-        <v>51.045</v>
-      </c>
-      <c r="M53" s="11" t="n">
-        <v>4.33</v>
+      <c r="L53" s="10" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="12" t="n">
+      <c r="A54" s="11" t="n">
         <v>50</v>
       </c>
-      <c r="B54" s="13" t="inlineStr">
+      <c r="B54" s="12" t="inlineStr">
         <is>
           <t>Protime (gruppo SD Worx)</t>
         </is>
       </c>
-      <c r="C54" s="13" t="inlineStr">
+      <c r="C54" s="12" t="inlineStr">
         <is>
           <t>Software HR</t>
         </is>
       </c>
-      <c r="D54" s="12" t="inlineStr">
+      <c r="D54" s="11" t="inlineStr">
         <is>
           <t>Kontichsesteenweg 54</t>
         </is>
       </c>
-      <c r="E54" s="12" t="inlineStr">
+      <c r="E54" s="11" t="inlineStr">
         <is>
           <t>Aartselaar</t>
         </is>
       </c>
-      <c r="F54" s="14" t="n">
+      <c r="F54" s="13" t="n">
         <v>8</v>
       </c>
-      <c r="G54" s="15" t="n">
+      <c r="G54" s="14" t="n">
         <v>376</v>
       </c>
-      <c r="H54" s="13" t="inlineStr">
+      <c r="H54" s="12" t="inlineStr">
         <is>
           <t>~376 dip. (gruppo)</t>
         </is>
       </c>
-      <c r="I54" s="12" t="inlineStr">
+      <c r="I54" s="11" t="inlineStr">
         <is>
           <t>info@protime.be</t>
         </is>
       </c>
-      <c r="J54" s="12" t="inlineStr"/>
-      <c r="K54" s="12" t="inlineStr">
+      <c r="J54" s="11" t="inlineStr"/>
+      <c r="K54" s="11" t="inlineStr">
         <is>
           <t>+32 3 870 60 30</t>
         </is>
       </c>
-      <c r="L54" s="16" t="n">
-        <v>51.138</v>
-      </c>
-      <c r="M54" s="16" t="n">
-        <v>4.399</v>
+      <c r="L54" s="15" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="7" t="n">
+      <c r="A55" s="6" t="n">
         <v>51</v>
       </c>
-      <c r="B55" s="8" t="inlineStr">
+      <c r="B55" s="7" t="inlineStr">
         <is>
           <t>Colis Privé BeLux</t>
         </is>
       </c>
-      <c r="C55" s="8" t="inlineStr">
+      <c r="C55" s="7" t="inlineStr">
         <is>
           <t>Pacchi/logistica</t>
         </is>
       </c>
-      <c r="D55" s="7" t="inlineStr">
+      <c r="D55" s="6" t="inlineStr">
         <is>
           <t>Schoondonkweg 4</t>
         </is>
       </c>
-      <c r="E55" s="7" t="inlineStr">
+      <c r="E55" s="6" t="inlineStr">
         <is>
           <t>Willebroek</t>
         </is>
       </c>
-      <c r="F55" s="9" t="n">
+      <c r="F55" s="8" t="n">
         <v>8.5</v>
       </c>
-      <c r="G55" s="10" t="n">
+      <c r="G55" s="9" t="n">
         <v>71</v>
       </c>
-      <c r="H55" s="8" t="inlineStr">
+      <c r="H55" s="7" t="inlineStr">
         <is>
           <t>71 FTE (companyweb)</t>
         </is>
       </c>
-      <c r="I55" s="7" t="inlineStr">
+      <c r="I55" s="6" t="inlineStr">
         <is>
           <t>infobelux@colisprive.com</t>
         </is>
       </c>
-      <c r="J55" s="7" t="inlineStr"/>
-      <c r="K55" s="7" t="inlineStr">
+      <c r="J55" s="6" t="inlineStr"/>
+      <c r="K55" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L55" s="11" t="n">
-        <v>51.051</v>
-      </c>
-      <c r="M55" s="11" t="n">
-        <v>4.372</v>
+      <c r="L55" s="10" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="12" t="n">
+      <c r="A56" s="11" t="n">
         <v>52</v>
       </c>
-      <c r="B56" s="13" t="inlineStr">
+      <c r="B56" s="12" t="inlineStr">
         <is>
           <t>PostNL – centro smistamento</t>
         </is>
       </c>
-      <c r="C56" s="13" t="inlineStr">
+      <c r="C56" s="12" t="inlineStr">
         <is>
           <t>Pacchi/logistica</t>
         </is>
       </c>
-      <c r="D56" s="12" t="inlineStr">
+      <c r="D56" s="11" t="inlineStr">
         <is>
           <t>MG Park De Hulst</t>
         </is>
       </c>
-      <c r="E56" s="12" t="inlineStr">
+      <c r="E56" s="11" t="inlineStr">
         <is>
           <t>Willebroek</t>
         </is>
       </c>
-      <c r="F56" s="14" t="n">
+      <c r="F56" s="13" t="n">
         <v>8.699999999999999</v>
       </c>
-      <c r="G56" s="15" t="n">
+      <c r="G56" s="14" t="n">
         <v>400</v>
       </c>
-      <c r="H56" s="13" t="inlineStr">
+      <c r="H56" s="12" t="inlineStr">
         <is>
           <t>~400 a regime, incl. 250 autisti (stampa)</t>
         </is>
       </c>
-      <c r="I56" s="18" t="inlineStr">
+      <c r="I56" s="17" t="inlineStr">
         <is>
           <t>n.d. (nessuna email locale pubblica)</t>
         </is>
       </c>
-      <c r="J56" s="12" t="inlineStr"/>
-      <c r="K56" s="12" t="inlineStr">
+      <c r="J56" s="11" t="inlineStr"/>
+      <c r="K56" s="11" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L56" s="16" t="n">
-        <v>51.05</v>
-      </c>
-      <c r="M56" s="16" t="n">
-        <v>4.375</v>
+      <c r="L56" s="15" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="7" t="n">
+      <c r="A57" s="6" t="n">
         <v>53</v>
       </c>
-      <c r="B57" s="8" t="inlineStr">
+      <c r="B57" s="7" t="inlineStr">
         <is>
           <t>Etex Building Performance (Promat)</t>
         </is>
       </c>
-      <c r="C57" s="8" t="inlineStr">
+      <c r="C57" s="7" t="inlineStr">
         <is>
           <t>Materiali edili – R&amp;D</t>
         </is>
       </c>
-      <c r="D57" s="7" t="inlineStr">
+      <c r="D57" s="6" t="inlineStr">
         <is>
           <t>Bormstraat 24</t>
         </is>
       </c>
-      <c r="E57" s="7" t="inlineStr">
+      <c r="E57" s="6" t="inlineStr">
         <is>
           <t>Willebroek (Tisselt)</t>
         </is>
       </c>
-      <c r="F57" s="9" t="n">
+      <c r="F57" s="8" t="n">
         <v>9.300000000000001</v>
       </c>
-      <c r="G57" s="10" t="n">
+      <c r="G57" s="9" t="n">
         <v>273</v>
       </c>
-      <c r="H57" s="8" t="inlineStr">
+      <c r="H57" s="7" t="inlineStr">
         <is>
           <t>273 FTE (companyweb)</t>
         </is>
       </c>
-      <c r="I57" s="7" t="inlineStr">
+      <c r="I57" s="6" t="inlineStr">
         <is>
           <t>info@promat.be</t>
         </is>
       </c>
-      <c r="J57" s="7" t="inlineStr"/>
-      <c r="K57" s="7" t="inlineStr">
+      <c r="J57" s="6" t="inlineStr"/>
+      <c r="K57" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L57" s="11" t="n">
-        <v>51.035</v>
-      </c>
-      <c r="M57" s="11" t="n">
-        <v>4.355</v>
+      <c r="L57" s="10" t="inlineStr">
+        <is>
+          <t>Apri percorso</t>
+        </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>Note: distanze in linea d'aria calcolate da coordinate stimate (±0,5–1 km); in auto aggiungere ~30–50%. Dipendenti = FTE dell'ultimo bilancio depositato (companyweb.be) salvo diversa indicazione. Email in rosso = nessun indirizzo generico pubblico: usare telefono/centralino o LinkedIn HR.</t>
+          <t>Note: distanza in linea d'aria da coordinate stimate (±0,5–1 km). Il link «Apri percorso» mostra su Google Maps km e tempo reali in auto (attenzione: Temse, Kruibeke e Hemiksem sono oltre la Schelda/Rupel, in auto il percorso è molto più lungo). Dipendenti = FTE dell'ultimo bilancio depositato (companyweb.be) salvo diversa indicazione. Email in rosso = nessun indirizzo generico pubblico: usare telefono/centralino o LinkedIn HR.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:M57"/>
+  <autoFilter ref="A4:L57"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L5" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L6" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L8" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L29" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L30" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L31" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L32" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L33" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L34" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L35" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L36" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L37" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L38" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L39" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L40" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L41" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L42" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L43" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L44" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L45" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L46" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L47" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L48" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L49" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L50" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L51" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L52" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L53" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L54" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L55" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L56" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L57" r:id="rId53"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -3517,152 +3491,152 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="19" t="inlineStr">
+      <c r="A1" s="18" t="inlineStr">
         <is>
           <t>Oggetto / Onderwerp:</t>
         </is>
       </c>
-      <c r="B1" s="20" t="inlineStr">
+      <c r="B1" s="19" t="inlineStr">
         <is>
           <t>Business lunch op een paar minuten van {bedrijf} – Arte Bianca Hingene</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="19" t="inlineStr"/>
-      <c r="B2" s="20" t="inlineStr"/>
+      <c r="A2" s="18" t="inlineStr"/>
+      <c r="B2" s="19" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="19" t="inlineStr">
+      <c r="A3" s="18" t="inlineStr">
         <is>
           <t>Testo:</t>
         </is>
       </c>
-      <c r="B3" s="20" t="inlineStr">
+      <c r="B3" s="19" t="inlineStr">
         <is>
           <t>Beste HR-team,</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="19" t="inlineStr"/>
-      <c r="B4" s="20" t="inlineStr"/>
+      <c r="A4" s="18" t="inlineStr"/>
+      <c r="B4" s="19" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="19" t="inlineStr"/>
-      <c r="B5" s="20" t="inlineStr">
+      <c r="A5" s="18" t="inlineStr"/>
+      <c r="B5" s="19" t="inlineStr">
         <is>
           <t>Wij zijn Arte Bianca, restaurant in de Egied De Jonghestraat 165 in Hingene (Bornem), op slechts {afstand} km van {bedrijf}.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="19" t="inlineStr"/>
-      <c r="B6" s="20" t="inlineStr"/>
+      <c r="A6" s="18" t="inlineStr"/>
+      <c r="B6" s="19" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="19" t="inlineStr"/>
-      <c r="B7" s="20" t="inlineStr">
+      <c r="A7" s="18" t="inlineStr"/>
+      <c r="B7" s="19" t="inlineStr">
         <is>
           <t>Voor bedrijven uit de buurt hebben we een business lunch: [menu/gerecht] voor €[prijs], vlot geserveerd zodat uw medewerkers binnen het uur terug op het werk zijn. Ideaal voor teamlunches, klantafspraken of als attentie voor uw personeel.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="19" t="inlineStr"/>
-      <c r="B8" s="20" t="inlineStr"/>
+      <c r="A8" s="18" t="inlineStr"/>
+      <c r="B8" s="19" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="19" t="inlineStr"/>
-      <c r="B9" s="20" t="inlineStr">
+      <c r="A9" s="18" t="inlineStr"/>
+      <c r="B9" s="19" t="inlineStr">
         <is>
           <t>Bekijk het menu: https://artebianca.be/business-lunch</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="inlineStr"/>
-      <c r="B10" s="20" t="inlineStr"/>
+      <c r="A10" s="18" t="inlineStr"/>
+      <c r="B10" s="19" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="inlineStr"/>
-      <c r="B11" s="20" t="inlineStr">
+      <c r="A11" s="18" t="inlineStr"/>
+      <c r="B11" s="19" t="inlineStr">
         <is>
           <t>Voor vaste groepen bieden we graag bedrijfsvoorwaarden aan (reservatie op vaste dagen, facturatie op bedrijfsnaam).</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="19" t="inlineStr"/>
-      <c r="B12" s="20" t="inlineStr">
+      <c r="A12" s="18" t="inlineStr"/>
+      <c r="B12" s="19" t="inlineStr">
         <is>
           <t>Mogen we u vragen dit door te sturen naar de collega's die teamactiviteiten of personeelsvoordelen organiseren?</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="19" t="inlineStr"/>
-      <c r="B13" s="20" t="inlineStr"/>
+      <c r="A13" s="18" t="inlineStr"/>
+      <c r="B13" s="19" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="19" t="inlineStr"/>
-      <c r="B14" s="20" t="inlineStr">
+      <c r="A14" s="18" t="inlineStr"/>
+      <c r="B14" s="19" t="inlineStr">
         <is>
           <t>Met vriendelijke groeten,</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="inlineStr"/>
-      <c r="B15" s="20" t="inlineStr">
+      <c r="A15" s="18" t="inlineStr"/>
+      <c r="B15" s="19" t="inlineStr">
         <is>
           <t>[Naam] – Arte Bianca</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="19" t="inlineStr"/>
-      <c r="B16" s="20" t="inlineStr">
+      <c r="A16" s="18" t="inlineStr"/>
+      <c r="B16" s="19" t="inlineStr">
         <is>
           <t>[telefoon] – artebianca.be</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="19" t="inlineStr"/>
-      <c r="B17" s="20" t="inlineStr"/>
+      <c r="A17" s="18" t="inlineStr"/>
+      <c r="B17" s="19" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="19" t="inlineStr"/>
-      <c r="B18" s="20" t="inlineStr">
+      <c r="A18" s="18" t="inlineStr"/>
+      <c r="B18" s="19" t="inlineStr">
         <is>
           <t>Wenst u geen berichten meer van ons te ontvangen? Antwoord met 'uitschrijven'.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="19" t="inlineStr"/>
-      <c r="B19" s="20" t="inlineStr"/>
+      <c r="A19" s="18" t="inlineStr"/>
+      <c r="B19" s="19" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="19" t="inlineStr">
+      <c r="A20" s="18" t="inlineStr">
         <is>
           <t>Uso:</t>
         </is>
       </c>
-      <c r="B20" s="20" t="inlineStr">
+      <c r="B20" s="19" t="inlineStr">
         <is>
           <t>Sostituisci {bedrijf} e {afstand} con le colonne B e F del foglio Aziende (stampa unione Gmail/Word). Invia in blocchi da 20–30/giorno per evitare lo spam.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="19" t="inlineStr">
+      <c r="A21" s="18" t="inlineStr">
         <is>
           <t>GDPR:</t>
         </is>
       </c>
-      <c r="B21" s="20" t="inlineStr">
+      <c r="B21" s="19" t="inlineStr">
         <is>
           <t>In Belgio le email B2B a indirizzi generici (info@, receptie@) sono ammesse senza consenso preventivo se pertinenti all'attività del destinatario e con possibilità di opt-out: lascia sempre la riga 'uitschrijven'.</t>
         </is>

</xml_diff>

<commit_message>
Fix NL outreach email template to match the takeaway business lunch offer
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JM7iB7irnbem4Sqp1rNjCu
</commit_message>
<xml_diff>
--- a/marketing/aziende_10km_arte_bianca.xlsx
+++ b/marketing/aziende_10km_arte_bianca.xlsx
@@ -3483,7 +3483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3498,7 +3498,7 @@
       </c>
       <c r="B1" s="19" t="inlineStr">
         <is>
-          <t>Business lunch op een paar minuten van {bedrijf} – Arte Bianca Hingene</t>
+          <t>Warme Italiaanse lunch voor uw team – op {afstand} km van {bedrijf}</t>
         </is>
       </c>
     </row>
@@ -3514,7 +3514,7 @@
       </c>
       <c r="B3" s="19" t="inlineStr">
         <is>
-          <t>Beste HR-team,</t>
+          <t>Goedemiddag,</t>
         </is>
       </c>
     </row>
@@ -3526,7 +3526,7 @@
       <c r="A5" s="18" t="inlineStr"/>
       <c r="B5" s="19" t="inlineStr">
         <is>
-          <t>Wij zijn Arte Bianca, restaurant in de Egied De Jonghestraat 165 in Hingene (Bornem), op slechts {afstand} km van {bedrijf}.</t>
+          <t>Op 8 oktober opent Arte Bianca in Wintam (Egied De Jonghestraat 165, Bornem), op {afstand} km van {bedrijf}.</t>
         </is>
       </c>
     </row>
@@ -3538,19 +3538,23 @@
       <c r="A7" s="18" t="inlineStr"/>
       <c r="B7" s="19" t="inlineStr">
         <is>
-          <t>Voor bedrijven uit de buurt hebben we een business lunch: [menu/gerecht] voor €[prijs], vlot geserveerd zodat uw medewerkers binnen het uur terug op het werk zijn. Ideaal voor teamlunches, klantafspraken of als attentie voor uw personeel.</t>
+          <t>Voor vergaderingen, opleidingen en teamlunches vanaf 10 personen:</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="18" t="inlineStr"/>
-      <c r="B8" s="19" t="inlineStr"/>
+      <c r="B8" s="19" t="inlineStr">
+        <is>
+          <t>- Menu Pizza: €18 p.p. – hele pizza, dessert en drank</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="18" t="inlineStr"/>
       <c r="B9" s="19" t="inlineStr">
         <is>
-          <t>Bekijk het menu: https://artebianca.be/business-lunch</t>
+          <t>- Menu Restaurant: €22 p.p. – lasagna, parmigiana of polpette met brood, dessert en drank</t>
         </is>
       </c>
     </row>
@@ -3562,83 +3566,103 @@
       <c r="A11" s="18" t="inlineStr"/>
       <c r="B11" s="19" t="inlineStr">
         <is>
-          <t>Voor vaste groepen bieden we graag bedrijfsvoorwaarden aan (reservatie op vaste dagen, facturatie op bedrijfsnaam).</t>
+          <t>Btw inbegrepen, warm verpakt, met allergenenlabels. U haalt af in Wintam tussen 11:30 en 13:00 (ma, di, do, vr, za). Bestellen 24–48 uur vooraf, één factuur.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="18" t="inlineStr"/>
-      <c r="B12" s="19" t="inlineStr">
-        <is>
-          <t>Mogen we u vragen dit door te sturen naar de collega's die teamactiviteiten of personeelsvoordelen organiseren?</t>
-        </is>
-      </c>
+      <c r="B12" s="19" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="18" t="inlineStr"/>
-      <c r="B13" s="19" t="inlineStr"/>
+      <c r="B13" s="19" t="inlineStr">
+        <is>
+          <t>Lanceringsaanbod tot 30 november: bij uw eerste bestelling is één menu gratis.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="18" t="inlineStr"/>
-      <c r="B14" s="19" t="inlineStr">
-        <is>
-          <t>Met vriendelijke groeten,</t>
-        </is>
-      </c>
+      <c r="B14" s="19" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="18" t="inlineStr"/>
       <c r="B15" s="19" t="inlineStr">
         <is>
-          <t>[Naam] – Arte Bianca</t>
+          <t>Wie organiseert bij u de lunch voor vergaderingen? We brengen graag een proefbox langs.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="18" t="inlineStr"/>
-      <c r="B16" s="19" t="inlineStr">
-        <is>
-          <t>[telefoon] – artebianca.be</t>
-        </is>
-      </c>
+      <c r="B16" s="19" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="18" t="inlineStr"/>
-      <c r="B17" s="19" t="inlineStr"/>
+      <c r="B17" s="19" t="inlineStr">
+        <is>
+          <t>Menu en bestellen: https://artebianca.be/nl/business-lunch/</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="18" t="inlineStr"/>
-      <c r="B18" s="19" t="inlineStr">
-        <is>
-          <t>Wenst u geen berichten meer van ons te ontvangen? Antwoord met 'uitschrijven'.</t>
-        </is>
-      </c>
+      <c r="B18" s="19" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="18" t="inlineStr"/>
-      <c r="B19" s="19" t="inlineStr"/>
+      <c r="B19" s="19" t="inlineStr">
+        <is>
+          <t>Met vriendelijke groet,</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="18" t="inlineStr">
+      <c r="A20" s="18" t="inlineStr"/>
+      <c r="B20" s="19" t="inlineStr">
+        <is>
+          <t>[naam] – Arte Bianca Wintam – +32 494 06 95 71</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="18" t="inlineStr"/>
+      <c r="B21" s="19" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="18" t="inlineStr"/>
+      <c r="B22" s="19" t="inlineStr">
+        <is>
+          <t>Geen berichten meer? Antwoord "uitschrijven".</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="18" t="inlineStr"/>
+      <c r="B23" s="19" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="18" t="inlineStr">
         <is>
           <t>Uso:</t>
         </is>
       </c>
-      <c r="B20" s="19" t="inlineStr">
-        <is>
-          <t>Sostituisci {bedrijf} e {afstand} con le colonne B e F del foglio Aziende (stampa unione Gmail/Word). Invia in blocchi da 20–30/giorno per evitare lo spam.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="18" t="inlineStr">
+      <c r="B24" s="19" t="inlineStr">
+        <is>
+          <t>Sostituisci {bedrijf} e {afstand} con le colonne B e F del foglio Aziende. Se non vuoi l'offerta di lancio, togli quella riga. Invia 20–30 email al giorno e richiama dopo 3 giorni.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="18" t="inlineStr">
         <is>
           <t>GDPR:</t>
         </is>
       </c>
-      <c r="B21" s="19" t="inlineStr">
-        <is>
-          <t>In Belgio le email B2B a indirizzi generici (info@, receptie@) sono ammesse senza consenso preventivo se pertinenti all'attività del destinatario e con possibilità di opt-out: lascia sempre la riga 'uitschrijven'.</t>
+      <c r="B25" s="19" t="inlineStr">
+        <is>
+          <t>Scrivi solo a indirizzi generici (info@, receptie@) e lascia sempre la riga 'uitschrijven'. Chi risponde 'uitschrijven' va tolto dalla lista.</t>
         </is>
       </c>
     </row>

</xml_diff>